<commit_message>
added CPT1 and CPT2 pathways
</commit_message>
<xml_diff>
--- a/pathway_pipeline/iembase-diseases-with-pathbank-pathways-and-hmdb-codes.xlsx
+++ b/pathway_pipeline/iembase-diseases-with-pathbank-pathways-and-hmdb-codes.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="530">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="531">
   <si>
     <t xml:space="preserve">Disease</t>
   </si>
@@ -608,6 +608,9 @@
   </si>
   <si>
     <t xml:space="preserve">Carnitine Palmitoyl Transferase Deficiency II </t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMP0658967</t>
   </si>
   <si>
     <t xml:space="preserve">L-Carnitine (HMDB0000062); Palmitoylcarnitine (HMDB0000222); Oleoylcarnitine (HMDB0005065)</t>
@@ -2693,1278 +2696,1281 @@
       <c r="E34" s="6" t="s">
         <v>194</v>
       </c>
+      <c r="F34" s="0" t="s">
+        <v>195</v>
+      </c>
       <c r="G34" s="0" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B35" s="1" t="n">
         <v>236200</v>
       </c>
       <c r="C35" s="0" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D35" s="0" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E35" s="0" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F35" s="0" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="G35" s="0" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C36" s="0" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D36" s="0" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E36" s="0" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F36" s="0" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="G36" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="0" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B37" s="1" t="n">
         <v>222748</v>
       </c>
       <c r="C37" s="0" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D37" s="0" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E37" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F37" s="0" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="G37" s="0" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="0" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B38" s="1" t="n">
         <v>274270</v>
       </c>
       <c r="C38" s="0" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D38" s="0" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E38" s="0" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="F38" s="0" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="G38" s="0" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C39" s="0" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D39" s="0" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E39" s="0" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="F39" s="0" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="G39" s="0" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C40" s="0" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D40" s="0" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E40" s="0" t="s">
         <v>36</v>
       </c>
       <c r="G40" s="0" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C41" s="0" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D41" s="0" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E41" s="0" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F41" s="0" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="G41" s="0" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C42" s="0" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D42" s="0" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="E42" s="0" t="s">
         <v>36</v>
       </c>
       <c r="G42" s="0" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C43" s="0" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D43" s="0" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E43" s="0" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="F43" s="0" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="G43" s="0" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="0" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C44" s="0" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D44" s="0" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E44" s="0" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="F44" s="0" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="G44" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B45" s="1" t="n">
         <v>606777</v>
       </c>
       <c r="C45" s="0" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D45" s="0" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E45" s="0" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="F45" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="G45" s="0" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="0" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C46" s="0" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D46" s="0" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E46" s="0" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="F46" s="0" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="G46" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="0" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B47" s="1" t="n">
         <v>231680</v>
       </c>
       <c r="C47" s="0" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D47" s="0" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E47" s="0" t="s">
         <v>36</v>
       </c>
       <c r="G47" s="0" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="0" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C48" s="0" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D48" s="0" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E48" s="0" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="F48" s="0" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="G48" s="0" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="0" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C49" s="0" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D49" s="0" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E49" s="0" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F49" s="0" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="G49" s="0" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="0" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C50" s="0" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D50" s="0" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E50" s="0" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F50" s="0" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="G50" s="0" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="0" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C51" s="0" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D51" s="0" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E51" s="0" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="F51" s="0" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="G51" s="0" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="0" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C52" s="0" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D52" s="0" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E52" s="0" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="F52" s="0" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="G52" s="0" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="0" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B53" s="1" t="n">
         <v>300322</v>
       </c>
       <c r="C53" s="0" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D53" s="0" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E53" s="0" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="F53" s="0" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="G53" s="0" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="0" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B54" s="1" t="n">
         <v>243500</v>
       </c>
       <c r="C54" s="0" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D54" s="0" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="E54" s="0" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="F54" s="0" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="G54" s="0" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="0" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B55" s="1" t="n">
         <v>609016</v>
       </c>
       <c r="C55" s="0" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D55" s="0" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="E55" s="0" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="F55" s="0" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="G55" s="0" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="0" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B56" s="1" t="n">
         <v>143450</v>
       </c>
       <c r="C56" s="0" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D56" s="0" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="E56" s="0" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="F56" s="0" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="G56" s="0" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="0" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B57" s="1" t="n">
         <v>222700</v>
       </c>
       <c r="C57" s="0" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="D57" s="0" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="E57" s="0" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="F57" s="0" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="G57" s="0" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="0" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B58" s="1" t="n">
         <v>248360</v>
       </c>
       <c r="C58" s="0" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="D58" s="0" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="E58" s="0" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="F58" s="0" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="G58" s="0" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="0" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B59" s="1" t="n">
         <v>248600</v>
       </c>
       <c r="C59" s="0" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="D59" s="0" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E59" s="0" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="F59" s="0" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="G59" s="0" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="0" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B60" s="1" t="n">
         <v>201450</v>
       </c>
       <c r="C60" s="0" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="D60" s="0" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E60" s="0" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="F60" s="0" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="G60" s="0" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="0" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B61" s="1" t="n">
         <v>250850</v>
       </c>
       <c r="C61" s="0" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="D61" s="0" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="E61" s="0" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="F61" s="0" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="G61" s="0" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="0" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B62" s="1" t="n">
         <v>251000</v>
       </c>
       <c r="C62" s="0" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="D62" s="0" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="E62" s="0" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="F62" s="0" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="G62" s="0" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="0" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B63" s="1" t="n">
         <v>251120</v>
       </c>
       <c r="C63" s="0" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="D63" s="0" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E63" s="0" t="s">
         <v>36</v>
       </c>
       <c r="G63" s="0" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="0" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="B64" s="1" t="n">
         <v>260920</v>
       </c>
       <c r="C64" s="0" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="D64" s="0" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="E64" s="0" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="F64" s="0" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="G64" s="0" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="0" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C65" s="0" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="D65" s="0" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="E65" s="0" t="s">
         <v>36</v>
       </c>
       <c r="G65" s="0" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="0" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B66" s="1" t="n">
         <v>252450</v>
       </c>
       <c r="C66" s="0" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="D66" s="0" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="E66" s="0" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="F66" s="0" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="G66" s="0" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="0" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B67" s="1" t="n">
         <v>611412</v>
       </c>
       <c r="C67" s="0" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="D67" s="0" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="E67" s="0" t="s">
         <v>36</v>
       </c>
       <c r="G67" s="0" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="0" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C68" s="0" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="D68" s="0" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E68" s="0" t="s">
         <v>36</v>
       </c>
       <c r="G68" s="0" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="0" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="C69" s="0" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="D69" s="0" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="E69" s="0" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="F69" s="0" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="G69" s="0" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="0" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="B70" s="1" t="n">
         <v>258870</v>
       </c>
       <c r="C70" s="0" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D70" s="0" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="E70" s="0" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="F70" s="0" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="G70" s="0" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="0" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B71" s="1" t="n">
         <v>311250</v>
       </c>
       <c r="C71" s="0" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="D71" s="0" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="E71" s="0" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="F71" s="0" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="G71" s="0" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="0" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="B72" s="1" t="n">
         <v>261600</v>
       </c>
       <c r="C72" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="D72" s="0" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="E72" s="0" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="F72" s="0" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="G72" s="0" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="0" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="B73" s="1" t="n">
         <v>170100</v>
       </c>
       <c r="C73" s="0" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="D73" s="0" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="E73" s="0" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="F73" s="0" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="G73" s="0" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="0" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="C74" s="0" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="D74" s="0" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="E74" s="0" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="F74" s="0" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="G74" s="0" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="0" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B75" s="1" t="n">
         <v>606054</v>
       </c>
       <c r="C75" s="0" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="D75" s="0" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="E75" s="0" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="F75" s="0" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="G75" s="0" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="0" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="B76" s="1" t="n">
         <v>266500</v>
       </c>
       <c r="C76" s="0" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="D76" s="0" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="E76" s="0" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="F76" s="0" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="G76" s="0" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="0" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="B77" s="1" t="n">
         <v>614707</v>
       </c>
       <c r="C77" s="0" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="D77" s="0" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="E77" s="0" t="s">
         <v>36</v>
       </c>
       <c r="G77" s="0" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="0" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="C78" s="0" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="D78" s="0" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="E78" s="0" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="F78" s="0" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="G78" s="0" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="0" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="C79" s="0" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="D79" s="0" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="E79" s="0" t="s">
         <v>36</v>
       </c>
       <c r="G79" s="0" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="0" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B80" s="1" t="n">
         <v>201470</v>
       </c>
       <c r="C80" s="0" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="D80" s="0" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="E80" s="0" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="F80" s="0" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="G80" s="0" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="0" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="B81" s="1" t="n">
         <v>600737</v>
       </c>
       <c r="C81" s="0" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="D81" s="0" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="E81" s="0" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="F81" s="0" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="G81" s="0" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="0" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="B82" s="1" t="n">
         <v>184420</v>
       </c>
       <c r="C82" s="0" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="D82" s="0" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="E82" s="0" t="s">
         <v>36</v>
       </c>
       <c r="G82" s="0" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="0" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="B83" s="1" t="n">
         <v>271980</v>
       </c>
       <c r="C83" s="0" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="D83" s="0" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="E83" s="0" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="F83" s="0" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="G83" s="0" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="0" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="B84" s="1" t="n">
         <v>606003</v>
       </c>
       <c r="C84" s="0" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="D84" s="0" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="E84" s="0" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="F84" s="0" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="G84" s="0" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="0" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="B85" s="1" t="n">
         <v>300872</v>
       </c>
       <c r="C85" s="0" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="D85" s="0" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="E85" s="0" t="s">
         <v>36</v>
       </c>
       <c r="G85" s="0" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="0" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="B86" s="1" t="n">
         <v>276700</v>
       </c>
       <c r="C86" s="0" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="D86" s="0" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="E86" s="0" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="F86" s="0" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="G86" s="0" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="0" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="B87" s="1" t="n">
         <v>258900</v>
       </c>
       <c r="C87" s="0" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="D87" s="0" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="E87" s="0" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="F87" s="0" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="G87" s="0" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="0" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="B88" s="1" t="n">
         <v>201475</v>
       </c>
       <c r="C88" s="0" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="D88" s="0" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="E88" s="0" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="F88" s="0" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="G88" s="0" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="0" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="B89" s="1" t="n">
         <v>603592</v>
       </c>
       <c r="C89" s="0" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="D89" s="0" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="E89" s="0" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="F89" s="0" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="G89" s="0" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="0" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="B90" s="1" t="n">
         <v>234580</v>
       </c>
       <c r="C90" s="0" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="D90" s="0" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="E90" s="0" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="F90" s="0" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="G90" s="0" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="0" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="0" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="0" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Frozen version with new adjustments to the disease pathway excel
</commit_message>
<xml_diff>
--- a/pathway_pipeline/iembase-diseases-with-pathbank-pathways-and-hmdb-codes.xlsx
+++ b/pathway_pipeline/iembase-diseases-with-pathbank-pathways-and-hmdb-codes.xlsx
@@ -11,7 +11,7 @@
     <sheet name="IEMbase_Diseases_with_Abbreviat" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">IEMbase_Diseases_with_Abbreviat!$A$1:$D$88</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">IEMbase_Diseases_with_Abbreviat!$A$1:$D$90</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="531">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="541">
   <si>
     <t xml:space="preserve">Disease</t>
   </si>
@@ -424,6 +424,24 @@
     <t xml:space="preserve">N-Acetylglycine (HMDB0000532); N-Acetylserine (HMDB0003011); N-Acetylglutamic acid (no HMDB entry found); N-Acetylglutamine (HMDB0006029); N-Acetyllysine (HMDB0000446); N-Acetylmethionine (HMDB0011745); N-Acetylvaline (HMDB0011757); N-Acetylleucine (HMDB0011756); N-Acetylisoleucine (HMDB0061684); N-Acetylasparagine (HMDB0006028)</t>
   </si>
   <si>
+    <t xml:space="preserve">Arginase deficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARG1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arginine ↑; Glutamine ↑; N-a-Acetyl-L-arginine ↑; Orotic acid ↑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Argininemia (Pathbank PW000138)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMP0120696</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arginine (HMDB0000517); Glutamine (HMDB0000641); N-a-Acetyl-L-arginine (HMDB0004620); Orotic acid (HMDB0000226)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Argininosuccinate lyase deficiency</t>
   </si>
   <si>
@@ -1457,6 +1475,18 @@
   </si>
   <si>
     <t xml:space="preserve">N-Acetylneuraminic acid (HMDB0000230)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLC22A5-related Primary carnitine deficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OCTN2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-carnitine ↓; Palmitoylcarnitine ↓; Stearoylcarnitine ↓; Oleoylcarnitine ↓</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-Carnitine (HMDB0000062); Palmitoylcarnitine (HMDB0000222); Stearoylcarnitine (HMDB0000848); Oleoylcarnitine (HMDB0005065)</t>
   </si>
   <si>
     <t xml:space="preserve">Squalene synthase deficiency</t>
@@ -1712,33 +1742,37 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1815,16 +1849,16 @@
         <a:srgbClr val="954f72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204" pitchFamily="0" charset="1"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="0" charset="1"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme>
@@ -1832,67 +1866,25 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:tint val="67000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:tint val="73000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:tint val="81000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:shade val="78000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:miter/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:miter/>
         </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:miter/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
@@ -1911,35 +1903,11 @@
           <a:schemeClr val="phClr"/>
         </a:solidFill>
         <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-          </a:schemeClr>
+          <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
@@ -1951,2030 +1919,2073 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G94"/>
+  <dimension ref="A1:G96"/>
   <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="23.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="196.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="80"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="15.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="23.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="196.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="80"/>
   </cols>
   <sheetData>
-    <row r="1" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="F2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="G2" s="1" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="1" t="n">
+      <c r="B3" s="2" t="n">
         <v>610006</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="E3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="F3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G3" s="0" t="s">
+      <c r="G3" s="1" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="0" t="s">
+      <c r="E4" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="F4" s="0" t="s">
+      <c r="F4" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="G4" s="0" t="s">
+      <c r="G4" s="1" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B5" s="1" t="n">
+      <c r="B5" s="2" t="n">
         <v>246450</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="0" t="s">
+      <c r="E5" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="F5" s="0" t="s">
+      <c r="F5" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="G5" s="0" t="s">
+      <c r="G5" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="1" t="n">
+      <c r="B6" s="2" t="n">
         <v>605197</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="E6" s="0" t="s">
+      <c r="E6" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G6" s="0" t="s">
+      <c r="G6" s="1" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B7" s="1" t="n">
+      <c r="B7" s="2" t="n">
         <v>203750</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D7" s="0" t="s">
+      <c r="D7" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="E7" s="0" t="s">
+      <c r="E7" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="F7" s="0" t="s">
+      <c r="F7" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="G7" s="0" t="s">
+      <c r="G7" s="1" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B8" s="1" t="n">
+      <c r="B8" s="2" t="n">
         <v>210200</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D8" s="0" t="s">
+      <c r="D8" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="E8" s="0" t="s">
+      <c r="E8" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="F8" s="0" t="s">
+      <c r="F8" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="G8" s="0" t="s">
+      <c r="G8" s="1" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B9" s="1" t="n">
+      <c r="B9" s="2" t="n">
         <v>613161</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D9" s="0" t="s">
+      <c r="D9" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="E9" s="0" t="s">
+      <c r="E9" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="F9" s="0" t="s">
+      <c r="F9" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="G9" s="0" t="s">
+      <c r="G9" s="1" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B10" s="1" t="n">
+      <c r="B10" s="2" t="n">
         <v>201810</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="C10" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D10" s="0" t="s">
+      <c r="D10" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="E10" s="0" t="s">
+      <c r="E10" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="F10" s="0" t="s">
+      <c r="F10" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="G10" s="0" t="s">
+      <c r="G10" s="1" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="C11" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="D11" s="0" t="s">
+      <c r="D11" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="E11" s="0" t="s">
+      <c r="E11" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="F11" s="0" t="s">
+      <c r="F11" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="G11" s="0" t="s">
+      <c r="G11" s="1" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="C12" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D12" s="0" t="s">
+      <c r="D12" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E12" s="0" t="s">
+      <c r="E12" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="F12" s="0" t="s">
+      <c r="F12" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="G12" s="0" t="s">
+      <c r="G12" s="1" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="C13" s="0" t="s">
+      <c r="C13" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="D13" s="0" t="s">
+      <c r="D13" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="E13" s="0" t="s">
+      <c r="E13" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G13" s="0" t="s">
+      <c r="G13" s="1" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C14" s="0" t="s">
+      <c r="C14" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="D14" s="0" t="s">
+      <c r="D14" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="E14" s="0" t="s">
+      <c r="E14" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G14" s="0" t="s">
+      <c r="G14" s="1" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+      <c r="A15" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="B15" s="1" t="n">
+      <c r="B15" s="2" t="n">
         <v>103050</v>
       </c>
-      <c r="C15" s="0" t="s">
+      <c r="C15" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="D15" s="0" t="s">
+      <c r="D15" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="E15" s="0" t="s">
+      <c r="E15" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="F15" s="0" t="s">
+      <c r="F15" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="G15" s="0" t="s">
+      <c r="G15" s="1" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="A16" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="B16" s="1" t="n">
+      <c r="B16" s="2" t="n">
         <v>608688</v>
       </c>
-      <c r="C16" s="0" t="s">
+      <c r="C16" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="D16" s="0" t="s">
+      <c r="D16" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="E16" s="0" t="s">
+      <c r="E16" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="F16" s="0" t="s">
+      <c r="F16" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="G16" s="0" t="s">
+      <c r="G16" s="1" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="B17" s="1" t="n">
+      <c r="B17" s="2" t="n">
         <v>266100</v>
       </c>
-      <c r="C17" s="0" t="s">
+      <c r="C17" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="D17" s="0" t="s">
+      <c r="D17" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="E17" s="0" t="s">
+      <c r="E17" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="F17" s="0" t="s">
+      <c r="F17" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="G17" s="0" t="s">
+      <c r="G17" s="1" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+      <c r="A18" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="C18" s="0" t="s">
+      <c r="C18" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="D18" s="0" t="s">
+      <c r="D18" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="E18" s="0" t="s">
+      <c r="E18" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="F18" s="0" t="s">
+      <c r="F18" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="G18" s="0" t="s">
+      <c r="G18" s="1" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+      <c r="A19" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="C19" s="0" t="s">
+      <c r="C19" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="D19" s="0" t="s">
+      <c r="D19" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="E19" s="0" t="s">
+      <c r="E19" s="1" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+      <c r="A20" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="C20" s="0" t="s">
+      <c r="C20" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D20" s="0" t="s">
+      <c r="D20" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="E20" s="0" t="s">
+      <c r="E20" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G20" s="0" t="s">
+      <c r="G20" s="1" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+      <c r="A21" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="C21" s="0" t="s">
+      <c r="C21" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="D21" s="0" t="s">
+      <c r="D21" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="E21" s="0" t="s">
+      <c r="E21" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G21" s="0" t="s">
+      <c r="G21" s="1" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
+      <c r="A22" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="C22" s="0" t="s">
+      <c r="C22" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="D22" s="0" t="s">
+      <c r="D22" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="E22" s="0" t="s">
+      <c r="E22" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G22" s="0" t="s">
+      <c r="G22" s="1" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
+      <c r="A23" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="B23" s="1" t="n">
+      <c r="B23" s="2" t="n">
         <v>609924</v>
       </c>
-      <c r="C23" s="0" t="s">
+      <c r="C23" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="D23" s="0" t="s">
+      <c r="D23" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="E23" s="0" t="s">
+      <c r="E23" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G23" s="0" t="s">
+      <c r="G23" s="1" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
+      <c r="A24" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B24" s="2" t="n">
+        <v>207800</v>
+      </c>
+      <c r="C24" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="C24" s="0" t="s">
+      <c r="D24" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="D24" s="0" t="s">
+      <c r="E24" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="E24" s="0" t="s">
+      <c r="F24" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="F24" s="0" t="s">
+      <c r="G24" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="G24" s="0" t="s">
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
+      <c r="B25" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="C25" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="C25" s="0" t="s">
+      <c r="D25" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="D25" s="0" t="s">
+      <c r="E25" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="E25" s="0" t="s">
+      <c r="F25" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="E26" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G25" s="0" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="s">
-        <v>145</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="C26" s="0" t="s">
-        <v>147</v>
-      </c>
-      <c r="D26" s="0" t="s">
-        <v>148</v>
-      </c>
-      <c r="E26" s="0" t="s">
+      <c r="G26" s="1" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="E27" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G26" s="0" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="s">
-        <v>150</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="C27" s="0" t="s">
-        <v>152</v>
-      </c>
-      <c r="D27" s="0" t="s">
-        <v>153</v>
-      </c>
-      <c r="E27" s="0" t="s">
+      <c r="G27" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="E28" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G27" s="0" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="s">
-        <v>155</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="C28" s="0" t="s">
-        <v>157</v>
-      </c>
-      <c r="D28" s="0" t="s">
-        <v>158</v>
-      </c>
-      <c r="E28" s="0" t="s">
+      <c r="G28" s="1" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="E29" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G28" s="0" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0" t="s">
-        <v>160</v>
-      </c>
-      <c r="B29" s="1" t="n">
+      <c r="G29" s="1" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="B30" s="2" t="n">
         <v>271900</v>
       </c>
-      <c r="C29" s="0" t="s">
-        <v>161</v>
-      </c>
-      <c r="D29" s="0" t="s">
-        <v>162</v>
-      </c>
-      <c r="E29" s="0" t="s">
-        <v>163</v>
-      </c>
-      <c r="F29" s="0" t="s">
-        <v>164</v>
-      </c>
-      <c r="G29" s="0" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0" t="s">
-        <v>166</v>
-      </c>
-      <c r="B30" s="1" t="s">
+      <c r="C30" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="C30" s="0" t="s">
+      <c r="D30" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="D30" s="0" t="s">
+      <c r="E30" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="E30" s="0" t="s">
+      <c r="F30" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="F30" s="0" t="s">
+      <c r="G30" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="G30" s="0" t="s">
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="1" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="s">
+      <c r="B31" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="B31" s="1" t="n">
+      <c r="C31" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="B32" s="2" t="n">
         <v>213700</v>
       </c>
-      <c r="C31" s="0" t="s">
-        <v>174</v>
-      </c>
-      <c r="D31" s="0" t="s">
-        <v>175</v>
-      </c>
-      <c r="E31" s="0" t="s">
-        <v>176</v>
-      </c>
-      <c r="F31" s="0" t="s">
-        <v>177</v>
-      </c>
-      <c r="G31" s="0" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="0" t="s">
-        <v>179</v>
-      </c>
-      <c r="B32" s="1" t="n">
+      <c r="C32" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="B33" s="2" t="n">
         <v>215700</v>
       </c>
-      <c r="C32" s="0" t="s">
-        <v>180</v>
-      </c>
-      <c r="D32" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="E32" s="0" t="s">
-        <v>182</v>
-      </c>
-      <c r="F32" s="0" t="s">
-        <v>183</v>
-      </c>
-      <c r="G32" s="0" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="B33" s="1" t="n">
+      <c r="C33" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="B34" s="2" t="n">
         <v>255120</v>
       </c>
-      <c r="C33" s="0" t="s">
-        <v>186</v>
-      </c>
-      <c r="D33" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="E33" s="0" t="s">
-        <v>188</v>
-      </c>
-      <c r="F33" s="0" t="s">
-        <v>189</v>
-      </c>
-      <c r="G33" s="0" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="0" t="s">
-        <v>191</v>
-      </c>
-      <c r="B34" s="1" t="n">
+      <c r="C34" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="B35" s="2" t="n">
         <v>255110</v>
       </c>
-      <c r="C34" s="0" t="s">
-        <v>192</v>
-      </c>
-      <c r="D34" s="5" t="s">
-        <v>193</v>
-      </c>
-      <c r="E34" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="F34" s="0" t="s">
-        <v>195</v>
-      </c>
-      <c r="G34" s="0" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="0" t="s">
-        <v>197</v>
-      </c>
-      <c r="B35" s="1" t="n">
+      <c r="C35" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="E35" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="B36" s="2" t="n">
         <v>236200</v>
       </c>
-      <c r="C35" s="0" t="s">
-        <v>198</v>
-      </c>
-      <c r="D35" s="0" t="s">
-        <v>199</v>
-      </c>
-      <c r="E35" s="0" t="s">
-        <v>200</v>
-      </c>
-      <c r="F35" s="0" t="s">
-        <v>201</v>
-      </c>
-      <c r="G35" s="0" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="0" t="s">
-        <v>203</v>
-      </c>
-      <c r="B36" s="1" t="s">
+      <c r="C36" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="C36" s="0" t="s">
+      <c r="D36" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="D36" s="0" t="s">
+      <c r="E36" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="E36" s="0" t="s">
+      <c r="F36" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="F36" s="0" t="s">
+      <c r="G36" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="G36" s="0" t="s">
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="1" t="s">
         <v>209</v>
       </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="0" t="s">
+      <c r="B37" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="B37" s="1" t="n">
+      <c r="C37" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="B38" s="2" t="n">
         <v>222748</v>
       </c>
-      <c r="C37" s="0" t="s">
-        <v>211</v>
-      </c>
-      <c r="D37" s="0" t="s">
-        <v>212</v>
-      </c>
-      <c r="E37" s="0" t="s">
-        <v>213</v>
-      </c>
-      <c r="F37" s="0" t="s">
-        <v>214</v>
-      </c>
-      <c r="G37" s="0" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="0" t="s">
-        <v>216</v>
-      </c>
-      <c r="B38" s="1" t="n">
+      <c r="C38" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="B39" s="2" t="n">
         <v>274270</v>
       </c>
-      <c r="C38" s="0" t="s">
-        <v>217</v>
-      </c>
-      <c r="D38" s="0" t="s">
-        <v>218</v>
-      </c>
-      <c r="E38" s="0" t="s">
-        <v>219</v>
-      </c>
-      <c r="F38" s="0" t="s">
-        <v>220</v>
-      </c>
-      <c r="G38" s="0" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="0" t="s">
-        <v>222</v>
-      </c>
-      <c r="B39" s="1" t="s">
+      <c r="C39" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="C39" s="0" t="s">
+      <c r="D39" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="D39" s="0" t="s">
+      <c r="E39" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="E39" s="0" t="s">
+      <c r="F39" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="F39" s="0" t="s">
+      <c r="G39" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="G39" s="0" t="s">
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="1" t="s">
         <v>228</v>
       </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="0" t="s">
+      <c r="B40" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="B40" s="1" t="s">
+      <c r="C40" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="C40" s="0" t="s">
+      <c r="D40" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="D40" s="0" t="s">
+      <c r="E40" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="E40" s="0" t="s">
+      <c r="F40" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="E41" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G40" s="0" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="0" t="s">
-        <v>234</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="C41" s="0" t="s">
-        <v>236</v>
-      </c>
-      <c r="D41" s="0" t="s">
-        <v>237</v>
-      </c>
-      <c r="E41" s="0" t="s">
-        <v>238</v>
-      </c>
-      <c r="F41" s="0" t="s">
+      <c r="G41" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="G41" s="0" t="s">
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="1" t="s">
         <v>240</v>
       </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="0" t="s">
+      <c r="B42" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="B42" s="1" t="s">
+      <c r="C42" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="C42" s="0" t="s">
+      <c r="D42" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="D42" s="0" t="s">
+      <c r="E42" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="E42" s="0" t="s">
+      <c r="F42" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="G42" s="1" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="E43" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G42" s="0" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="0" t="s">
-        <v>246</v>
-      </c>
-      <c r="B43" s="1" t="s">
-        <v>247</v>
-      </c>
-      <c r="C43" s="0" t="s">
-        <v>248</v>
-      </c>
-      <c r="D43" s="0" t="s">
-        <v>249</v>
-      </c>
-      <c r="E43" s="0" t="s">
-        <v>250</v>
-      </c>
-      <c r="F43" s="0" t="s">
+      <c r="G43" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="G43" s="0" t="s">
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="1" t="s">
         <v>252</v>
       </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="0" t="s">
+      <c r="B44" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="B44" s="1" t="s">
+      <c r="C44" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="C44" s="0" t="s">
+      <c r="D44" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="D44" s="0" t="s">
+      <c r="E44" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="E44" s="0" t="s">
+      <c r="F44" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="F44" s="0" t="s">
+      <c r="G44" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="G44" s="0" t="s">
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="1" t="s">
         <v>259</v>
       </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="0" t="s">
+      <c r="B45" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="B45" s="1" t="n">
+      <c r="C45" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="G45" s="1" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="B46" s="2" t="n">
         <v>606777</v>
       </c>
-      <c r="C45" s="0" t="s">
-        <v>261</v>
-      </c>
-      <c r="D45" s="0" t="s">
+      <c r="C46" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="D47" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="E45" s="0" t="s">
-        <v>263</v>
-      </c>
-      <c r="F45" s="0" t="s">
-        <v>264</v>
-      </c>
-      <c r="G45" s="0" t="s">
+      <c r="E47" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="G47" s="1" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="0" t="s">
-        <v>266</v>
-      </c>
-      <c r="B46" s="1" t="s">
-        <v>267</v>
-      </c>
-      <c r="C46" s="0" t="s">
-        <v>268</v>
-      </c>
-      <c r="D46" s="0" t="s">
-        <v>256</v>
-      </c>
-      <c r="E46" s="0" t="s">
-        <v>269</v>
-      </c>
-      <c r="F46" s="0" t="s">
-        <v>270</v>
-      </c>
-      <c r="G46" s="0" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="0" t="s">
-        <v>271</v>
-      </c>
-      <c r="B47" s="1" t="n">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="B48" s="2" t="n">
         <v>231680</v>
       </c>
-      <c r="C47" s="0" t="s">
-        <v>272</v>
-      </c>
-      <c r="D47" s="0" t="s">
-        <v>273</v>
-      </c>
-      <c r="E47" s="0" t="s">
+      <c r="C48" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="E48" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G47" s="0" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="0" t="s">
-        <v>275</v>
-      </c>
-      <c r="B48" s="1" t="s">
-        <v>276</v>
-      </c>
-      <c r="C48" s="0" t="s">
-        <v>277</v>
-      </c>
-      <c r="D48" s="0" t="s">
-        <v>278</v>
-      </c>
-      <c r="E48" s="0" t="s">
-        <v>279</v>
-      </c>
-      <c r="F48" s="0" t="s">
+      <c r="G48" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="G48" s="0" t="s">
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="1" t="s">
         <v>281</v>
       </c>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="0" t="s">
+      <c r="B49" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="B49" s="1" t="s">
+      <c r="C49" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="C49" s="0" t="s">
+      <c r="D49" s="1" t="s">
         <v>284</v>
       </c>
-      <c r="D49" s="0" t="s">
+      <c r="E49" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="E49" s="0" t="s">
+      <c r="F49" s="1" t="s">
         <v>286</v>
       </c>
-      <c r="F49" s="0" t="s">
+      <c r="G49" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="G49" s="0" t="s">
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="1" t="s">
         <v>288</v>
       </c>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="0" t="s">
+      <c r="B50" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="B50" s="1" t="s">
+      <c r="C50" s="1" t="s">
         <v>290</v>
       </c>
-      <c r="C50" s="0" t="s">
+      <c r="D50" s="1" t="s">
         <v>291</v>
       </c>
-      <c r="D50" s="0" t="s">
+      <c r="E50" s="1" t="s">
         <v>292</v>
       </c>
-      <c r="E50" s="0" t="s">
+      <c r="F50" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="F50" s="0" t="s">
+      <c r="G50" s="1" t="s">
         <v>294</v>
       </c>
-      <c r="G50" s="0" t="s">
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="1" t="s">
         <v>295</v>
       </c>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="0" t="s">
+      <c r="B51" s="2" t="s">
         <v>296</v>
       </c>
-      <c r="B51" s="1" t="s">
+      <c r="C51" s="1" t="s">
         <v>297</v>
       </c>
-      <c r="C51" s="0" t="s">
+      <c r="D51" s="1" t="s">
         <v>298</v>
       </c>
-      <c r="D51" s="0" t="s">
+      <c r="E51" s="1" t="s">
         <v>299</v>
       </c>
-      <c r="E51" s="0" t="s">
+      <c r="F51" s="1" t="s">
         <v>300</v>
       </c>
-      <c r="F51" s="0" t="s">
+      <c r="G51" s="1" t="s">
         <v>301</v>
       </c>
-      <c r="G51" s="0" t="s">
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="1" t="s">
         <v>302</v>
       </c>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="0" t="s">
+      <c r="B52" s="2" t="s">
         <v>303</v>
       </c>
-      <c r="B52" s="1" t="s">
+      <c r="C52" s="1" t="s">
         <v>304</v>
       </c>
-      <c r="C52" s="0" t="s">
+      <c r="D52" s="1" t="s">
         <v>305</v>
       </c>
-      <c r="D52" s="0" t="s">
+      <c r="E52" s="1" t="s">
         <v>306</v>
       </c>
-      <c r="E52" s="0" t="s">
+      <c r="F52" s="1" t="s">
         <v>307</v>
       </c>
-      <c r="F52" s="0" t="s">
+      <c r="G52" s="1" t="s">
         <v>308</v>
       </c>
-      <c r="G52" s="0" t="s">
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="1" t="s">
         <v>309</v>
       </c>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="0" t="s">
+      <c r="B53" s="2" t="s">
         <v>310</v>
       </c>
-      <c r="B53" s="1" t="n">
+      <c r="C53" s="1" t="s">
+        <v>311</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="E53" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="F53" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="G53" s="1" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="B54" s="2" t="n">
         <v>300322</v>
       </c>
-      <c r="C53" s="0" t="s">
-        <v>311</v>
-      </c>
-      <c r="D53" s="0" t="s">
-        <v>312</v>
-      </c>
-      <c r="E53" s="0" t="s">
-        <v>313</v>
-      </c>
-      <c r="F53" s="0" t="s">
-        <v>314</v>
-      </c>
-      <c r="G53" s="0" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="0" t="s">
-        <v>316</v>
-      </c>
-      <c r="B54" s="1" t="n">
+      <c r="C54" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="G54" s="1" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="1" t="s">
+        <v>322</v>
+      </c>
+      <c r="B55" s="2" t="n">
         <v>243500</v>
       </c>
-      <c r="C54" s="0" t="s">
-        <v>317</v>
-      </c>
-      <c r="D54" s="0" t="s">
-        <v>318</v>
-      </c>
-      <c r="E54" s="0" t="s">
-        <v>319</v>
-      </c>
-      <c r="F54" s="0" t="s">
-        <v>320</v>
-      </c>
-      <c r="G54" s="0" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="0" t="s">
-        <v>322</v>
-      </c>
-      <c r="B55" s="1" t="n">
+      <c r="C55" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="G55" s="1" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="B56" s="2" t="n">
         <v>609016</v>
       </c>
-      <c r="C55" s="0" t="s">
-        <v>323</v>
-      </c>
-      <c r="D55" s="0" t="s">
-        <v>324</v>
-      </c>
-      <c r="E55" s="0" t="s">
-        <v>325</v>
-      </c>
-      <c r="F55" s="0" t="s">
-        <v>326</v>
-      </c>
-      <c r="G55" s="0" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="0" t="s">
-        <v>328</v>
-      </c>
-      <c r="B56" s="1" t="n">
+      <c r="C56" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F56" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="G56" s="1" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="B57" s="2" t="n">
         <v>143450</v>
       </c>
-      <c r="C56" s="0" t="s">
-        <v>329</v>
-      </c>
-      <c r="D56" s="0" t="s">
-        <v>330</v>
-      </c>
-      <c r="E56" s="0" t="s">
-        <v>331</v>
-      </c>
-      <c r="F56" s="0" t="s">
-        <v>332</v>
-      </c>
-      <c r="G56" s="0" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="0" t="s">
-        <v>334</v>
-      </c>
-      <c r="B57" s="1" t="n">
+      <c r="C57" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="F57" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="G57" s="1" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="B58" s="2" t="n">
         <v>222700</v>
       </c>
-      <c r="C57" s="0" t="s">
-        <v>335</v>
-      </c>
-      <c r="D57" s="0" t="s">
-        <v>336</v>
-      </c>
-      <c r="E57" s="0" t="s">
-        <v>337</v>
-      </c>
-      <c r="F57" s="0" t="s">
-        <v>338</v>
-      </c>
-      <c r="G57" s="0" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="0" t="s">
-        <v>340</v>
-      </c>
-      <c r="B58" s="1" t="n">
+      <c r="C58" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>343</v>
+      </c>
+      <c r="F58" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="G58" s="1" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="1" t="s">
+        <v>346</v>
+      </c>
+      <c r="B59" s="2" t="n">
         <v>248360</v>
       </c>
-      <c r="C58" s="0" t="s">
-        <v>341</v>
-      </c>
-      <c r="D58" s="0" t="s">
-        <v>342</v>
-      </c>
-      <c r="E58" s="0" t="s">
-        <v>343</v>
-      </c>
-      <c r="F58" s="0" t="s">
-        <v>344</v>
-      </c>
-      <c r="G58" s="0" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="0" t="s">
-        <v>346</v>
-      </c>
-      <c r="B59" s="1" t="n">
+      <c r="C59" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="E59" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="G59" s="1" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="1" t="s">
+        <v>352</v>
+      </c>
+      <c r="B60" s="2" t="n">
         <v>248600</v>
       </c>
-      <c r="C59" s="0" t="s">
-        <v>347</v>
-      </c>
-      <c r="D59" s="0" t="s">
-        <v>348</v>
-      </c>
-      <c r="E59" s="0" t="s">
-        <v>349</v>
-      </c>
-      <c r="F59" s="0" t="s">
-        <v>350</v>
-      </c>
-      <c r="G59" s="0" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="0" t="s">
-        <v>352</v>
-      </c>
-      <c r="B60" s="1" t="n">
+      <c r="C60" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="F60" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="G60" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B61" s="2" t="n">
         <v>201450</v>
       </c>
-      <c r="C60" s="0" t="s">
-        <v>353</v>
-      </c>
-      <c r="D60" s="0" t="s">
-        <v>354</v>
-      </c>
-      <c r="E60" s="0" t="s">
-        <v>355</v>
-      </c>
-      <c r="F60" s="0" t="s">
-        <v>356</v>
-      </c>
-      <c r="G60" s="0" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="0" t="s">
-        <v>358</v>
-      </c>
-      <c r="B61" s="1" t="n">
+      <c r="C61" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="D61" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="E61" s="1" t="s">
+        <v>361</v>
+      </c>
+      <c r="F61" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="G61" s="1" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="B62" s="2" t="n">
         <v>250850</v>
       </c>
-      <c r="C61" s="0" t="s">
-        <v>359</v>
-      </c>
-      <c r="D61" s="0" t="s">
-        <v>360</v>
-      </c>
-      <c r="E61" s="0" t="s">
-        <v>361</v>
-      </c>
-      <c r="F61" s="0" t="s">
-        <v>362</v>
-      </c>
-      <c r="G61" s="0" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="0" t="s">
-        <v>364</v>
-      </c>
-      <c r="B62" s="1" t="n">
+      <c r="C62" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="E62" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="F62" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="G62" s="1" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="B63" s="2" t="n">
         <v>251000</v>
       </c>
-      <c r="C62" s="0" t="s">
-        <v>365</v>
-      </c>
-      <c r="D62" s="0" t="s">
-        <v>366</v>
-      </c>
-      <c r="E62" s="0" t="s">
-        <v>367</v>
-      </c>
-      <c r="F62" s="0" t="s">
-        <v>368</v>
-      </c>
-      <c r="G62" s="0" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="0" t="s">
-        <v>370</v>
-      </c>
-      <c r="B63" s="1" t="n">
+      <c r="C63" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="D63" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="E63" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="F63" s="1" t="s">
+        <v>374</v>
+      </c>
+      <c r="G63" s="1" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="1" t="s">
+        <v>376</v>
+      </c>
+      <c r="B64" s="2" t="n">
         <v>251120</v>
       </c>
-      <c r="C63" s="0" t="s">
-        <v>371</v>
-      </c>
-      <c r="D63" s="0" t="s">
-        <v>372</v>
-      </c>
-      <c r="E63" s="0" t="s">
+      <c r="C64" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="D64" s="1" t="s">
+        <v>378</v>
+      </c>
+      <c r="E64" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G63" s="0" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="0" t="s">
-        <v>374</v>
-      </c>
-      <c r="B64" s="1" t="n">
+      <c r="G64" s="1" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="B65" s="2" t="n">
         <v>260920</v>
       </c>
-      <c r="C64" s="0" t="s">
-        <v>375</v>
-      </c>
-      <c r="D64" s="0" t="s">
-        <v>376</v>
-      </c>
-      <c r="E64" s="0" t="s">
-        <v>377</v>
-      </c>
-      <c r="F64" s="0" t="s">
-        <v>378</v>
-      </c>
-      <c r="G64" s="0" t="s">
-        <v>379</v>
-      </c>
-    </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="0" t="s">
-        <v>380</v>
-      </c>
-      <c r="B65" s="1" t="s">
+      <c r="C65" s="1" t="s">
         <v>381</v>
       </c>
-      <c r="C65" s="0" t="s">
+      <c r="D65" s="1" t="s">
         <v>382</v>
       </c>
-      <c r="D65" s="0" t="s">
+      <c r="E65" s="1" t="s">
         <v>383</v>
       </c>
-      <c r="E65" s="0" t="s">
+      <c r="F65" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="G65" s="1" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="1" t="s">
+        <v>386</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="D66" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="E66" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G65" s="0" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="0" t="s">
-        <v>385</v>
-      </c>
-      <c r="B66" s="1" t="n">
+      <c r="G66" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="1" t="s">
+        <v>391</v>
+      </c>
+      <c r="B67" s="2" t="n">
         <v>252450</v>
       </c>
-      <c r="C66" s="0" t="s">
-        <v>386</v>
-      </c>
-      <c r="D66" s="0" t="s">
-        <v>387</v>
-      </c>
-      <c r="E66" s="0" t="s">
-        <v>388</v>
-      </c>
-      <c r="F66" s="0" t="s">
-        <v>389</v>
-      </c>
-      <c r="G66" s="0" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="0" t="s">
-        <v>391</v>
-      </c>
-      <c r="B67" s="1" t="n">
+      <c r="C67" s="1" t="s">
+        <v>392</v>
+      </c>
+      <c r="D67" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="E67" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="F67" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="G67" s="1" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="1" t="s">
+        <v>397</v>
+      </c>
+      <c r="B68" s="2" t="n">
         <v>611412</v>
       </c>
-      <c r="C67" s="0" t="s">
-        <v>392</v>
-      </c>
-      <c r="D67" s="0" t="s">
-        <v>393</v>
-      </c>
-      <c r="E67" s="0" t="s">
+      <c r="C68" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="D68" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="E68" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G67" s="0" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="0" t="s">
-        <v>395</v>
-      </c>
-      <c r="B68" s="1" t="s">
-        <v>396</v>
-      </c>
-      <c r="C68" s="0" t="s">
-        <v>397</v>
-      </c>
-      <c r="D68" s="0" t="s">
-        <v>398</v>
-      </c>
-      <c r="E68" s="0" t="s">
+      <c r="G68" s="1" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="1" t="s">
+        <v>401</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="D69" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="E69" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G68" s="0" t="s">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="0" t="s">
-        <v>400</v>
-      </c>
-      <c r="B69" s="1" t="s">
-        <v>401</v>
-      </c>
-      <c r="C69" s="0" t="s">
-        <v>402</v>
-      </c>
-      <c r="D69" s="0" t="s">
-        <v>403</v>
-      </c>
-      <c r="E69" s="0" t="s">
-        <v>404</v>
-      </c>
-      <c r="F69" s="0" t="s">
+      <c r="G69" s="1" t="s">
         <v>405</v>
       </c>
-      <c r="G69" s="0" t="s">
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="1" t="s">
         <v>406</v>
       </c>
-    </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="0" t="s">
+      <c r="B70" s="2" t="s">
         <v>407</v>
       </c>
-      <c r="B70" s="1" t="n">
+      <c r="C70" s="1" t="s">
+        <v>408</v>
+      </c>
+      <c r="D70" s="1" t="s">
+        <v>409</v>
+      </c>
+      <c r="E70" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="F70" s="1" t="s">
+        <v>411</v>
+      </c>
+      <c r="G70" s="1" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="B71" s="2" t="n">
         <v>258870</v>
       </c>
-      <c r="C70" s="0" t="s">
-        <v>408</v>
-      </c>
-      <c r="D70" s="0" t="s">
-        <v>409</v>
-      </c>
-      <c r="E70" s="0" t="s">
-        <v>410</v>
-      </c>
-      <c r="F70" s="0" t="s">
-        <v>411</v>
-      </c>
-      <c r="G70" s="0" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="71" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A71" s="0" t="s">
-        <v>413</v>
-      </c>
-      <c r="B71" s="1" t="n">
+      <c r="C71" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="D71" s="1" t="s">
+        <v>415</v>
+      </c>
+      <c r="E71" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="F71" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="G71" s="1" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A72" s="1" t="s">
+        <v>419</v>
+      </c>
+      <c r="B72" s="2" t="n">
         <v>311250</v>
       </c>
-      <c r="C71" s="0" t="s">
-        <v>414</v>
-      </c>
-      <c r="D71" s="0" t="s">
-        <v>415</v>
-      </c>
-      <c r="E71" s="0" t="s">
-        <v>416</v>
-      </c>
-      <c r="F71" s="0" t="s">
-        <v>417</v>
-      </c>
-      <c r="G71" s="0" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="0" t="s">
-        <v>419</v>
-      </c>
-      <c r="B72" s="1" t="n">
+      <c r="C72" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="D72" s="1" t="s">
+        <v>421</v>
+      </c>
+      <c r="E72" s="1" t="s">
+        <v>422</v>
+      </c>
+      <c r="F72" s="1" t="s">
+        <v>423</v>
+      </c>
+      <c r="G72" s="1" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A73" s="1" t="s">
+        <v>425</v>
+      </c>
+      <c r="B73" s="2" t="n">
         <v>261600</v>
       </c>
-      <c r="C72" s="0" t="s">
-        <v>420</v>
-      </c>
-      <c r="D72" s="0" t="s">
-        <v>421</v>
-      </c>
-      <c r="E72" s="0" t="s">
-        <v>422</v>
-      </c>
-      <c r="F72" s="0" t="s">
-        <v>423</v>
-      </c>
-      <c r="G72" s="0" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="0" t="s">
-        <v>425</v>
-      </c>
-      <c r="B73" s="1" t="n">
+      <c r="C73" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="D73" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="E73" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="F73" s="1" t="s">
+        <v>429</v>
+      </c>
+      <c r="G73" s="1" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="B74" s="2" t="n">
         <v>170100</v>
       </c>
-      <c r="C73" s="0" t="s">
-        <v>426</v>
-      </c>
-      <c r="D73" s="0" t="s">
-        <v>427</v>
-      </c>
-      <c r="E73" s="0" t="s">
-        <v>428</v>
-      </c>
-      <c r="F73" s="0" t="s">
-        <v>429</v>
-      </c>
-      <c r="G73" s="0" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="0" t="s">
-        <v>431</v>
-      </c>
-      <c r="B74" s="1" t="s">
+      <c r="C74" s="1" t="s">
         <v>432</v>
       </c>
-      <c r="C74" s="0" t="s">
+      <c r="D74" s="1" t="s">
         <v>433</v>
       </c>
-      <c r="D74" s="0" t="s">
+      <c r="E74" s="1" t="s">
         <v>434</v>
       </c>
-      <c r="E74" s="0" t="s">
+      <c r="F74" s="1" t="s">
         <v>435</v>
       </c>
-      <c r="F74" s="0" t="s">
+      <c r="G74" s="1" t="s">
         <v>436</v>
       </c>
-      <c r="G74" s="0" t="s">
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="1" t="s">
         <v>437</v>
       </c>
-    </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="0" t="s">
+      <c r="B75" s="2" t="s">
         <v>438</v>
       </c>
-      <c r="B75" s="1" t="n">
+      <c r="C75" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="D75" s="1" t="s">
+        <v>440</v>
+      </c>
+      <c r="E75" s="1" t="s">
+        <v>441</v>
+      </c>
+      <c r="F75" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="G75" s="1" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="B76" s="2" t="n">
         <v>606054</v>
       </c>
-      <c r="C75" s="0" t="s">
-        <v>439</v>
-      </c>
-      <c r="D75" s="0" t="s">
-        <v>440</v>
-      </c>
-      <c r="E75" s="0" t="s">
-        <v>441</v>
-      </c>
-      <c r="F75" s="0" t="s">
-        <v>442</v>
-      </c>
-      <c r="G75" s="0" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="0" t="s">
-        <v>444</v>
-      </c>
-      <c r="B76" s="1" t="n">
+      <c r="C76" s="1" t="s">
+        <v>445</v>
+      </c>
+      <c r="D76" s="1" t="s">
+        <v>446</v>
+      </c>
+      <c r="E76" s="1" t="s">
+        <v>447</v>
+      </c>
+      <c r="F76" s="1" t="s">
+        <v>448</v>
+      </c>
+      <c r="G76" s="1" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="B77" s="2" t="n">
         <v>266500</v>
       </c>
-      <c r="C76" s="0" t="s">
-        <v>445</v>
-      </c>
-      <c r="D76" s="0" t="s">
-        <v>446</v>
-      </c>
-      <c r="E76" s="0" t="s">
-        <v>447</v>
-      </c>
-      <c r="F76" s="0" t="s">
-        <v>448</v>
-      </c>
-      <c r="G76" s="0" t="s">
-        <v>449</v>
-      </c>
-    </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="0" t="s">
-        <v>450</v>
-      </c>
-      <c r="B77" s="1" t="n">
+      <c r="C77" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="D77" s="1" t="s">
+        <v>452</v>
+      </c>
+      <c r="E77" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="F77" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="G77" s="1" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="B78" s="2" t="n">
         <v>614707</v>
       </c>
-      <c r="C77" s="0" t="s">
-        <v>451</v>
-      </c>
-      <c r="D77" s="0" t="s">
-        <v>452</v>
-      </c>
-      <c r="E77" s="0" t="s">
+      <c r="C78" s="1" t="s">
+        <v>457</v>
+      </c>
+      <c r="D78" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="E78" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G77" s="0" t="s">
-        <v>453</v>
-      </c>
-    </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="0" t="s">
-        <v>454</v>
-      </c>
-      <c r="B78" s="1" t="s">
-        <v>455</v>
-      </c>
-      <c r="C78" s="0" t="s">
-        <v>456</v>
-      </c>
-      <c r="D78" s="0" t="s">
-        <v>457</v>
-      </c>
-      <c r="E78" s="0" t="s">
-        <v>458</v>
-      </c>
-      <c r="F78" s="0" t="s">
+      <c r="G78" s="1" t="s">
         <v>459</v>
       </c>
-      <c r="G78" s="0" t="s">
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="1" t="s">
         <v>460</v>
       </c>
-    </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="0" t="s">
+      <c r="B79" s="2" t="s">
         <v>461</v>
       </c>
-      <c r="B79" s="1" t="s">
+      <c r="C79" s="1" t="s">
         <v>462</v>
       </c>
-      <c r="C79" s="0" t="s">
+      <c r="D79" s="1" t="s">
         <v>463</v>
       </c>
-      <c r="D79" s="0" t="s">
+      <c r="E79" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="E79" s="0" t="s">
+      <c r="F79" s="1" t="s">
+        <v>465</v>
+      </c>
+      <c r="G79" s="1" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>468</v>
+      </c>
+      <c r="C80" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="D80" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="E80" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G79" s="0" t="s">
-        <v>465</v>
-      </c>
-    </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="0" t="s">
-        <v>466</v>
-      </c>
-      <c r="B80" s="1" t="n">
+      <c r="G80" s="1" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="B81" s="2" t="n">
         <v>201470</v>
       </c>
-      <c r="C80" s="0" t="s">
-        <v>467</v>
-      </c>
-      <c r="D80" s="0" t="s">
-        <v>468</v>
-      </c>
-      <c r="E80" s="0" t="s">
-        <v>469</v>
-      </c>
-      <c r="F80" s="0" t="s">
-        <v>470</v>
-      </c>
-      <c r="G80" s="0" t="s">
-        <v>471</v>
-      </c>
-    </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="0" t="s">
-        <v>472</v>
-      </c>
-      <c r="B81" s="1" t="n">
+      <c r="C81" s="1" t="s">
+        <v>473</v>
+      </c>
+      <c r="D81" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="E81" s="1" t="s">
+        <v>475</v>
+      </c>
+      <c r="F81" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="G81" s="1" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="B82" s="2" t="n">
         <v>600737</v>
       </c>
-      <c r="C81" s="0" t="s">
-        <v>473</v>
-      </c>
-      <c r="D81" s="0" t="s">
-        <v>474</v>
-      </c>
-      <c r="E81" s="0" t="s">
-        <v>475</v>
-      </c>
-      <c r="F81" s="0" t="s">
-        <v>476</v>
-      </c>
-      <c r="G81" s="0" t="s">
-        <v>477</v>
-      </c>
-    </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="0" t="s">
-        <v>478</v>
-      </c>
-      <c r="B82" s="1" t="n">
+      <c r="C82" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="D82" s="1" t="s">
+        <v>480</v>
+      </c>
+      <c r="E82" s="1" t="s">
+        <v>481</v>
+      </c>
+      <c r="F82" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="G82" s="1" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="B83" s="2" t="n">
+        <v>212140</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="D83" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="E83" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G83" s="1" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="B84" s="2" t="n">
         <v>184420</v>
       </c>
-      <c r="C82" s="0" t="s">
-        <v>479</v>
-      </c>
-      <c r="D82" s="0" t="s">
-        <v>480</v>
-      </c>
-      <c r="E82" s="0" t="s">
+      <c r="C84" s="1" t="s">
+        <v>489</v>
+      </c>
+      <c r="D84" s="1" t="s">
+        <v>490</v>
+      </c>
+      <c r="E84" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G82" s="0" t="s">
-        <v>481</v>
-      </c>
-    </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="0" t="s">
-        <v>482</v>
-      </c>
-      <c r="B83" s="1" t="n">
+      <c r="G84" s="1" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="B85" s="2" t="n">
         <v>271980</v>
       </c>
-      <c r="C83" s="0" t="s">
-        <v>483</v>
-      </c>
-      <c r="D83" s="0" t="s">
-        <v>484</v>
-      </c>
-      <c r="E83" s="0" t="s">
-        <v>485</v>
-      </c>
-      <c r="F83" s="0" t="s">
-        <v>486</v>
-      </c>
-      <c r="G83" s="0" t="s">
-        <v>487</v>
-      </c>
-    </row>
-    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="0" t="s">
-        <v>488</v>
-      </c>
-      <c r="B84" s="1" t="n">
+      <c r="C85" s="1" t="s">
+        <v>493</v>
+      </c>
+      <c r="D85" s="1" t="s">
+        <v>494</v>
+      </c>
+      <c r="E85" s="1" t="s">
+        <v>495</v>
+      </c>
+      <c r="F85" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="G85" s="1" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="1" t="s">
+        <v>498</v>
+      </c>
+      <c r="B86" s="2" t="n">
         <v>606003</v>
       </c>
-      <c r="C84" s="0" t="s">
-        <v>489</v>
-      </c>
-      <c r="D84" s="0" t="s">
-        <v>490</v>
-      </c>
-      <c r="E84" s="0" t="s">
-        <v>491</v>
-      </c>
-      <c r="F84" s="0" t="s">
-        <v>492</v>
-      </c>
-      <c r="G84" s="0" t="s">
-        <v>493</v>
-      </c>
-    </row>
-    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="0" t="s">
-        <v>494</v>
-      </c>
-      <c r="B85" s="1" t="n">
+      <c r="C86" s="1" t="s">
+        <v>499</v>
+      </c>
+      <c r="D86" s="1" t="s">
+        <v>500</v>
+      </c>
+      <c r="E86" s="1" t="s">
+        <v>501</v>
+      </c>
+      <c r="F86" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="G86" s="1" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="1" t="s">
+        <v>504</v>
+      </c>
+      <c r="B87" s="2" t="n">
         <v>300872</v>
       </c>
-      <c r="C85" s="0" t="s">
-        <v>495</v>
-      </c>
-      <c r="D85" s="0" t="s">
-        <v>496</v>
-      </c>
-      <c r="E85" s="0" t="s">
+      <c r="C87" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="D87" s="1" t="s">
+        <v>506</v>
+      </c>
+      <c r="E87" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G85" s="0" t="s">
-        <v>497</v>
-      </c>
-    </row>
-    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="0" t="s">
-        <v>498</v>
-      </c>
-      <c r="B86" s="1" t="n">
+      <c r="G87" s="1" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="1" t="s">
+        <v>508</v>
+      </c>
+      <c r="B88" s="2" t="n">
         <v>276700</v>
       </c>
-      <c r="C86" s="0" t="s">
-        <v>499</v>
-      </c>
-      <c r="D86" s="0" t="s">
-        <v>500</v>
-      </c>
-      <c r="E86" s="0" t="s">
-        <v>501</v>
-      </c>
-      <c r="F86" s="0" t="s">
-        <v>502</v>
-      </c>
-      <c r="G86" s="0" t="s">
-        <v>503</v>
-      </c>
-    </row>
-    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="0" t="s">
-        <v>504</v>
-      </c>
-      <c r="B87" s="1" t="n">
+      <c r="C88" s="1" t="s">
+        <v>509</v>
+      </c>
+      <c r="D88" s="1" t="s">
+        <v>510</v>
+      </c>
+      <c r="E88" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="F88" s="1" t="s">
+        <v>512</v>
+      </c>
+      <c r="G88" s="1" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="1" t="s">
+        <v>514</v>
+      </c>
+      <c r="B89" s="2" t="n">
         <v>258900</v>
       </c>
-      <c r="C87" s="0" t="s">
-        <v>505</v>
-      </c>
-      <c r="D87" s="0" t="s">
-        <v>506</v>
-      </c>
-      <c r="E87" s="0" t="s">
-        <v>507</v>
-      </c>
-      <c r="F87" s="0" t="s">
-        <v>508</v>
-      </c>
-      <c r="G87" s="0" t="s">
-        <v>509</v>
-      </c>
-    </row>
-    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="0" t="s">
-        <v>510</v>
-      </c>
-      <c r="B88" s="1" t="n">
+      <c r="C89" s="1" t="s">
+        <v>515</v>
+      </c>
+      <c r="D89" s="1" t="s">
+        <v>516</v>
+      </c>
+      <c r="E89" s="1" t="s">
+        <v>517</v>
+      </c>
+      <c r="F89" s="1" t="s">
+        <v>518</v>
+      </c>
+      <c r="G89" s="1" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="1" t="s">
+        <v>520</v>
+      </c>
+      <c r="B90" s="2" t="n">
         <v>201475</v>
       </c>
-      <c r="C88" s="0" t="s">
-        <v>511</v>
-      </c>
-      <c r="D88" s="0" t="s">
-        <v>512</v>
-      </c>
-      <c r="E88" s="0" t="s">
-        <v>513</v>
-      </c>
-      <c r="F88" s="0" t="s">
-        <v>514</v>
-      </c>
-      <c r="G88" s="0" t="s">
-        <v>515</v>
-      </c>
-    </row>
-    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="0" t="s">
-        <v>516</v>
-      </c>
-      <c r="B89" s="1" t="n">
+      <c r="C90" s="1" t="s">
+        <v>521</v>
+      </c>
+      <c r="D90" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="E90" s="1" t="s">
+        <v>523</v>
+      </c>
+      <c r="F90" s="1" t="s">
+        <v>524</v>
+      </c>
+      <c r="G90" s="1" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="1" t="s">
+        <v>526</v>
+      </c>
+      <c r="B91" s="2" t="n">
         <v>603592</v>
       </c>
-      <c r="C89" s="0" t="s">
-        <v>517</v>
-      </c>
-      <c r="D89" s="0" t="s">
-        <v>518</v>
-      </c>
-      <c r="E89" s="0" t="s">
-        <v>519</v>
-      </c>
-      <c r="F89" s="0" t="s">
-        <v>520</v>
-      </c>
-      <c r="G89" s="0" t="s">
-        <v>521</v>
-      </c>
-    </row>
-    <row r="90" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A90" s="0" t="s">
-        <v>522</v>
-      </c>
-      <c r="B90" s="1" t="n">
+      <c r="C91" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="D91" s="1" t="s">
+        <v>528</v>
+      </c>
+      <c r="E91" s="1" t="s">
+        <v>529</v>
+      </c>
+      <c r="F91" s="1" t="s">
+        <v>530</v>
+      </c>
+      <c r="G91" s="1" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A92" s="1" t="s">
+        <v>532</v>
+      </c>
+      <c r="B92" s="2" t="n">
         <v>234580</v>
       </c>
-      <c r="C90" s="0" t="s">
-        <v>523</v>
-      </c>
-      <c r="D90" s="0" t="s">
-        <v>524</v>
-      </c>
-      <c r="E90" s="0" t="s">
-        <v>525</v>
-      </c>
-      <c r="F90" s="0" t="s">
-        <v>526</v>
-      </c>
-      <c r="G90" s="0" t="s">
-        <v>527</v>
-      </c>
-    </row>
-    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="0" t="s">
-        <v>528</v>
-      </c>
-    </row>
-    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="0" t="s">
-        <v>529</v>
+      <c r="C92" s="1" t="s">
+        <v>533</v>
+      </c>
+      <c r="D92" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="E92" s="1" t="s">
+        <v>535</v>
+      </c>
+      <c r="F92" s="1" t="s">
+        <v>536</v>
+      </c>
+      <c r="G92" s="1" t="s">
+        <v>537</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="0" t="s">
-        <v>530</v>
+      <c r="A94" s="1" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="1" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="1" t="s">
+        <v>540</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D88"/>
+  <autoFilter ref="A1:D90"/>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" display="236792; 600721"/>
   </hyperlinks>

</xml_diff>

<commit_message>
Changed disease iembase excel
</commit_message>
<xml_diff>
--- a/pathway_pipeline/iembase-diseases-with-pathbank-pathways-and-hmdb-codes.xlsx
+++ b/pathway_pipeline/iembase-diseases-with-pathbank-pathways-and-hmdb-codes.xlsx
@@ -11,7 +11,7 @@
     <sheet name="IEMbase_Diseases_with_Abbreviat" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">IEMbase_Diseases_with_Abbreviat!$A$1:$D$90</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">IEMbase_Diseases_with_Abbreviat!$A$1:$D$91</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="541">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="545">
   <si>
     <t xml:space="preserve">Disease</t>
   </si>
@@ -325,7 +325,7 @@
     <t xml:space="preserve">AASADHD</t>
   </si>
   <si>
-    <t xml:space="preserve">2,3,4,5-Tetrahydropiperidine-2-carboxylate (P6C) ↑; Allysine ↑; Pipecolic acid ↑; 6-oxoPIP ↑; 2-OPP ↑; 6-CMP ↑</t>
+    <t xml:space="preserve">2,3,4,5-Tetrahydropiperidine-2-carboxylate (P6C) ↑; Allysine ↑; Pipecolic acid ↑; 6-Oxo-pipecolinic acid ↑; 2-oxopropylpiperidine-2-carboxylic acid ↑; (2S,6S)-6-(carboxymethyl)piperidine-w-carboxylic acid ↑</t>
   </si>
   <si>
     <t xml:space="preserve">Pyridoxine Dependency with Seizures (PathBank PW000547)</t>
@@ -334,7 +334,7 @@
     <t xml:space="preserve">SMP0000571</t>
   </si>
   <si>
-    <t xml:space="preserve">2,3,4,5-Tetrahydropiperidine-2-carboxylate (P6C) (no HMDB entry found); Allysine (HMDB0001263); Pipecolic acid (HMDB0000716); 6-oxoPIP (HMDB0061705); 2-OPP (no HMDB entry found); 6-CMP (no HMDB entry found)</t>
+    <t xml:space="preserve">2,3,4,5-Tetrahydropiperidine-2-carboxylate (P6C) (no HMDB entry found); Allysine (HMDB0001263); Pipecolic acid (HMDB0000716); 6-Oxo-pipecolinic acid (HMDB0061705); 2-oxopropylpiperidine-2-carboxylic acid (HMDB0341532) ; (2S,6S)-6-(carboxymethyl)piperidine-w-carboxylic acid (HMDB0340289) </t>
   </si>
   <si>
     <t xml:space="preserve">Alpha-aminoadipic semialdehyde synthase deficiency</t>
@@ -355,7 +355,7 @@
     <t xml:space="preserve">SMP0000719</t>
   </si>
   <si>
-    <t xml:space="preserve">Lysine (HMDB0000182); N-Acetyllysine (HMDB0000446); Pipecolic acid (HMDB0000716); Homocitrulline (no HMDB entry found)</t>
+    <t xml:space="preserve">Lysine (HMDB0000182); N-Acetyllysine (HMDB0000446); Pipecolic acid (HMDB0000716); Homocitrulline (HMDB0000679)</t>
   </si>
   <si>
     <t xml:space="preserve">Aminocarboxymuconate semialdehyde decarboxylase deficiency</t>
@@ -421,7 +421,7 @@
     <t xml:space="preserve">N-Acetylglycine ↑; N-Acetylserine ↑; N-Acetylglutamic acid ↑; N-Acetylglutamine ↑; N-Acetyllysine ↑; N-Acetylmethionine ↑; N-Acetylvaline ↑; N-Acetylleucine ↑; N-Acetylisoleucine ↑; N-Acetylasparagine ↑</t>
   </si>
   <si>
-    <t xml:space="preserve">N-Acetylglycine (HMDB0000532); N-Acetylserine (HMDB0003011); N-Acetylglutamic acid (no HMDB entry found); N-Acetylglutamine (HMDB0006029); N-Acetyllysine (HMDB0000446); N-Acetylmethionine (HMDB0011745); N-Acetylvaline (HMDB0011757); N-Acetylleucine (HMDB0011756); N-Acetylisoleucine (HMDB0061684); N-Acetylasparagine (HMDB0006028)</t>
+    <t xml:space="preserve">N-Acetylglycine (HMDB0000532); N-Acetylserine (HMDB0003011); N-Acetylglutamic acid (HMDB0001138); N-Acetylglutamine (HMDB0006029); N-Acetyllysine (HMDB0000446); N-Acetylmethionine (HMDB0011745); N-Acetylvaline (HMDB0011757); N-Acetylleucine (HMDB0011756); N-Acetylisoleucine (HMDB0061684); N-Acetylasparagine (HMDB0006028)</t>
   </si>
   <si>
     <t xml:space="preserve">Arginase deficiency</t>
@@ -451,7 +451,7 @@
     <t xml:space="preserve">ASLD</t>
   </si>
   <si>
-    <t xml:space="preserve">Cirulline ↑; N-Acetylcitrulline ↑; Uridine ↑; Cytidine ↑; Argininosuccinic acid ↑; Homocitrulline ↑</t>
+    <t xml:space="preserve">Cirulline ↑; N-Acetylcitrulline ↑; Uridine ↑; Cytidine ↑; Argininosuccinic acid ↑; Homocitrulline ↑; Arginine ↓</t>
   </si>
   <si>
     <t xml:space="preserve">Argininosuccinic Aciduria (PathBank PW000184)</t>
@@ -460,7 +460,7 @@
     <t xml:space="preserve">SMP0000003</t>
   </si>
   <si>
-    <t xml:space="preserve">Cirulline (HMDB0000904); N-Acetylcitrulline (HMDB0000856); Uridine (HMDB0000296); Cytidine (HMDB0000089); Argininosuccinic acid (HMDB0000052); Homocitrulline (no HMDB entry found)</t>
+    <t xml:space="preserve">Cirulline (HMDB0000904); N-Acetylcitrulline (HMDB0000856); Uridine (HMDB0000296); Cytidine (HMDB0000089); Argininosuccinic acid (HMDB0000052); Homocitrulline (HMDB0000679); Arginine (HMDB0000517)</t>
   </si>
   <si>
     <t xml:space="preserve">Aromatic l-amino acid decarboxylase deficiency</t>
@@ -490,7 +490,7 @@
     <t xml:space="preserve">N-Acetylaspartic acid ↓*; N-Acetylaspartylglutamate ↓*</t>
   </si>
   <si>
-    <t xml:space="preserve">N-Acetylaspartic acid (no HMDB entry found); N-Acetylaspartylglutamate (no HMDB entry found)</t>
+    <t xml:space="preserve">N-Acetyl-L-aspartic acid (HMDB0000812); N-Acetylaspartylglutamate (HMDB0001067)</t>
   </si>
   <si>
     <t xml:space="preserve">Aspartylglucosaminidase deficiency</t>
@@ -538,7 +538,7 @@
     <t xml:space="preserve">SMP0000175</t>
   </si>
   <si>
-    <t xml:space="preserve">N-Acetylaspartic acid (no HMDB entry found)</t>
+    <t xml:space="preserve">N-Acetyl-L-aspartic acid (HMDB0000812)</t>
   </si>
   <si>
     <t xml:space="preserve">Carbamoyl-phosphate synthetase I deficiency</t>
@@ -580,13 +580,25 @@
     <t xml:space="preserve">Cholestane-pentol (HMDB0002208); Cholestane-glucuronides (no HMDB entry found)</t>
   </si>
   <si>
+    <t xml:space="preserve">Citrin deficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CTLN2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Citrulline ↑; Arginine ↑; Glutamine ↑; Threonine ↑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arginine (HMDB0000517); Citrulline (HMDB0000904); Glutamine (HMDB0000641); Threonine (HMDB0000167)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Citrullinemia</t>
   </si>
   <si>
     <t xml:space="preserve">CTLN1</t>
   </si>
   <si>
-    <t xml:space="preserve">Citrulline ↑; N-Acetylcitrulline ↑</t>
+    <t xml:space="preserve">Citrulline ↑; N-Acetylcitrulline ↑; Arginine ↓</t>
   </si>
   <si>
     <t xml:space="preserve">Citrullinemia Type I (PathBank PW000185)</t>
@@ -595,7 +607,7 @@
     <t xml:space="preserve">SMP0000001</t>
   </si>
   <si>
-    <t xml:space="preserve">Citrulline (HMDB0000904); N-Acetylcitrulline (HMDB0000856)</t>
+    <t xml:space="preserve">Citrulline (HMDB0000904); N-Acetylcitrulline (HMDB0000856); Arginine (HMDB0000517)</t>
   </si>
   <si>
     <t xml:space="preserve">CPT1A deficiency</t>
@@ -640,7 +652,7 @@
     <t xml:space="preserve">CBS </t>
   </si>
   <si>
-    <t xml:space="preserve">Methionine ↑; Glutamyl-methionine ↑; Methionine-hexose ↑; 5'-Methylthioadenosine ↑</t>
+    <t xml:space="preserve">Methionine ↑; Glutamyl-methionine ↑; Methionine-hexose ↑; 5'-Methylthioadenosine ↑; Homocysteine ↑</t>
   </si>
   <si>
     <t xml:space="preserve">Cystathionine beta-Synthase Deficiency (PathBank PW000100)</t>
@@ -649,7 +661,7 @@
     <t xml:space="preserve">SMP0000177</t>
   </si>
   <si>
-    <t xml:space="preserve">Methionine (HMDB0000696); Glutamyl-methionine (HMDB0034367); Methionine-hexose (no HMDB entry found); 5'-Methylthioadenosine (HMDB0001173)</t>
+    <t xml:space="preserve">Methionine (HMDB0000696); Glutamyl-methionine (HMDB0034367); Methionine-hexose (no HMDB entry found); 5'-Methylthioadenosine (HMDB0001173); Homocysteine (HMDB0000742)</t>
   </si>
   <si>
     <t xml:space="preserve">Cytosolic phosphoenolpyruvate carboxykinase deficiency</t>
@@ -970,7 +982,7 @@
     <t xml:space="preserve">SMP0000360</t>
   </si>
   <si>
-    <t xml:space="preserve">Proline (HMDB0000162); Pyrrole-2-carboxylic acid (HMDB0004230); 2-Pyrroloylglycine (no HMDB entry found); Pyrrole-2-carboxylic acid (HMDB0004230); (2 R)-5-(2-oxopropyl)pyrrolidine-2-carboxylic acid (no HMDB entry found); (2 R)-5-(carboxymethyl)pyrrolidine-2-carboxylic acid (no HMDB entry found)</t>
+    <t xml:space="preserve">Proline (HMDB0000162); Pyrrole-2-carboxylic acid (HMDB0004230); 2-Pyrroloylglycine (HMDB0059778); Pyrrole-2-carboxylic acid (HMDB0004230); (2 R)-5-(2-oxopropyl)pyrrolidine-2-carboxylic acid (no HMDB entry found); (2 R)-5-(carboxymethyl)pyrrolidine-2-carboxylic acid (no HMDB entry found)</t>
   </si>
   <si>
     <t xml:space="preserve">Hypoxanthine guanine phosphoribosyltransferase deficiency</t>
@@ -1655,7 +1667,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1692,12 +1704,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1742,7 +1748,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1761,10 +1767,6 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -1919,7 +1921,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G96"/>
+  <dimension ref="A1:G97"/>
   <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="51"/>
@@ -2512,7 +2514,7 @@
       <c r="E27" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G27" s="1" t="s">
+      <c r="G27" s="5" t="s">
         <v>155</v>
       </c>
     </row>
@@ -2630,720 +2632,720 @@
         <v>185</v>
       </c>
       <c r="B33" s="2" t="n">
-        <v>215700</v>
+        <v>603859</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="D33" s="6" t="s">
+      <c r="D33" s="5" t="s">
         <v>187</v>
       </c>
       <c r="E33" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G33" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="F33" s="1" t="s">
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="G33" s="1" t="s">
+      <c r="B34" s="2" t="n">
+        <v>215700</v>
+      </c>
+      <c r="C34" s="1" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="7" t="s">
+      <c r="D34" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="B34" s="2" t="n">
+      <c r="E34" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="B35" s="2" t="n">
         <v>255120</v>
       </c>
-      <c r="C34" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="D34" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="G34" s="1" t="s">
+      <c r="C35" s="1" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="1" t="s">
+      <c r="D35" s="5" t="s">
         <v>197</v>
       </c>
-      <c r="B35" s="2" t="n">
-        <v>255110</v>
-      </c>
-      <c r="C35" s="1" t="s">
+      <c r="E35" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="D35" s="7" t="s">
+      <c r="F35" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="E35" s="6" t="s">
+      <c r="G35" s="1" t="s">
         <v>200</v>
-      </c>
-      <c r="F35" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="G35" s="1" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="B36" s="2" t="n">
+        <v>255110</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="D36" s="6" t="s">
         <v>203</v>
       </c>
-      <c r="B36" s="2" t="n">
-        <v>236200</v>
-      </c>
-      <c r="C36" s="1" t="s">
+      <c r="E36" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="D36" s="1" t="s">
+      <c r="F36" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="E36" s="1" t="s">
+      <c r="G36" s="1" t="s">
         <v>206</v>
-      </c>
-      <c r="F36" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="G36" s="1" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="B37" s="2" t="n">
+        <v>236200</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="D37" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="E37" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="C37" s="1" t="s">
+      <c r="F37" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="D37" s="1" t="s">
+      <c r="G37" s="1" t="s">
         <v>212</v>
-      </c>
-      <c r="E37" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>214</v>
-      </c>
-      <c r="G37" s="1" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="D38" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="B38" s="2" t="n">
-        <v>222748</v>
-      </c>
-      <c r="C38" s="1" t="s">
+      <c r="E38" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="D38" s="1" t="s">
+      <c r="F38" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="E38" s="1" t="s">
+      <c r="G38" s="1" t="s">
         <v>219</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>220</v>
-      </c>
-      <c r="G38" s="1" t="s">
-        <v>221</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="B39" s="2" t="n">
+        <v>222748</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="D39" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="B39" s="2" t="n">
-        <v>274270</v>
-      </c>
-      <c r="C39" s="1" t="s">
+      <c r="E39" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="D39" s="1" t="s">
+      <c r="F39" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="E39" s="1" t="s">
+      <c r="G39" s="1" t="s">
         <v>225</v>
-      </c>
-      <c r="F39" s="1" t="s">
-        <v>226</v>
-      </c>
-      <c r="G39" s="1" t="s">
-        <v>227</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="B40" s="2" t="n">
+        <v>274270</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="D40" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="E40" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="C40" s="1" t="s">
+      <c r="F40" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="D40" s="1" t="s">
+      <c r="G40" s="1" t="s">
         <v>231</v>
-      </c>
-      <c r="E40" s="1" t="s">
-        <v>232</v>
-      </c>
-      <c r="F40" s="1" t="s">
-        <v>233</v>
-      </c>
-      <c r="G40" s="1" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="D41" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="B41" s="2" t="s">
+      <c r="E41" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="C41" s="1" t="s">
+      <c r="F41" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="D41" s="1" t="s">
+      <c r="G41" s="1" t="s">
         <v>238</v>
-      </c>
-      <c r="E41" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="G41" s="1" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="B42" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="C42" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="C42" s="1" t="s">
+      <c r="D42" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="D42" s="1" t="s">
+      <c r="E42" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G42" s="1" t="s">
         <v>243</v>
-      </c>
-      <c r="E42" s="1" t="s">
-        <v>244</v>
-      </c>
-      <c r="F42" s="1" t="s">
-        <v>245</v>
-      </c>
-      <c r="G42" s="1" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D43" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="B43" s="2" t="s">
+      <c r="E43" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="C43" s="1" t="s">
+      <c r="F43" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="D43" s="1" t="s">
+      <c r="G43" s="1" t="s">
         <v>250</v>
-      </c>
-      <c r="E43" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="G43" s="1" t="s">
-        <v>251</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="B44" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="C44" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="C44" s="1" t="s">
+      <c r="D44" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="D44" s="1" t="s">
+      <c r="E44" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G44" s="1" t="s">
         <v>255</v>
-      </c>
-      <c r="E44" s="1" t="s">
-        <v>256</v>
-      </c>
-      <c r="F44" s="1" t="s">
-        <v>257</v>
-      </c>
-      <c r="G44" s="1" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="D45" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="B45" s="2" t="s">
+      <c r="E45" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="C45" s="1" t="s">
+      <c r="F45" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="D45" s="1" t="s">
+      <c r="G45" s="1" t="s">
         <v>262</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>263</v>
-      </c>
-      <c r="F45" s="1" t="s">
-        <v>264</v>
-      </c>
-      <c r="G45" s="1" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="D46" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="B46" s="2" t="n">
-        <v>606777</v>
-      </c>
-      <c r="C46" s="1" t="s">
+      <c r="E46" s="1" t="s">
         <v>267</v>
       </c>
-      <c r="D46" s="1" t="s">
+      <c r="F46" s="1" t="s">
         <v>268</v>
       </c>
-      <c r="E46" s="1" t="s">
+      <c r="G46" s="1" t="s">
         <v>269</v>
-      </c>
-      <c r="F46" s="1" t="s">
-        <v>270</v>
-      </c>
-      <c r="G46" s="1" t="s">
-        <v>271</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="B47" s="2" t="n">
+        <v>606777</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="D47" s="1" t="s">
         <v>272</v>
       </c>
-      <c r="B47" s="2" t="s">
+      <c r="E47" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="C47" s="1" t="s">
+      <c r="F47" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="D47" s="1" t="s">
-        <v>262</v>
-      </c>
-      <c r="E47" s="1" t="s">
+      <c r="G47" s="1" t="s">
         <v>275</v>
-      </c>
-      <c r="F47" s="1" t="s">
-        <v>276</v>
-      </c>
-      <c r="G47" s="1" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="B48" s="2" t="s">
         <v>277</v>
-      </c>
-      <c r="B48" s="2" t="n">
-        <v>231680</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>278</v>
       </c>
       <c r="D48" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="E48" s="1" t="s">
         <v>279</v>
       </c>
-      <c r="E48" s="1" t="s">
-        <v>36</v>
+      <c r="F48" s="1" t="s">
+        <v>280</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>280</v>
+        <v>269</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="B49" s="2" t="s">
+      <c r="B49" s="2" t="n">
+        <v>231680</v>
+      </c>
+      <c r="C49" s="1" t="s">
         <v>282</v>
       </c>
-      <c r="C49" s="1" t="s">
+      <c r="D49" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="D49" s="1" t="s">
+      <c r="E49" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G49" s="1" t="s">
         <v>284</v>
-      </c>
-      <c r="E49" s="1" t="s">
-        <v>285</v>
-      </c>
-      <c r="F49" s="1" t="s">
-        <v>286</v>
-      </c>
-      <c r="G49" s="1" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="D50" s="1" t="s">
         <v>288</v>
       </c>
-      <c r="B50" s="2" t="s">
+      <c r="E50" s="1" t="s">
         <v>289</v>
       </c>
-      <c r="C50" s="1" t="s">
+      <c r="F50" s="1" t="s">
         <v>290</v>
       </c>
-      <c r="D50" s="1" t="s">
+      <c r="G50" s="1" t="s">
         <v>291</v>
-      </c>
-      <c r="E50" s="1" t="s">
-        <v>292</v>
-      </c>
-      <c r="F50" s="1" t="s">
-        <v>293</v>
-      </c>
-      <c r="G50" s="1" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="D51" s="1" t="s">
         <v>295</v>
       </c>
-      <c r="B51" s="2" t="s">
+      <c r="E51" s="1" t="s">
         <v>296</v>
       </c>
-      <c r="C51" s="1" t="s">
+      <c r="F51" s="1" t="s">
         <v>297</v>
       </c>
-      <c r="D51" s="1" t="s">
+      <c r="G51" s="1" t="s">
         <v>298</v>
-      </c>
-      <c r="E51" s="1" t="s">
-        <v>299</v>
-      </c>
-      <c r="F51" s="1" t="s">
-        <v>300</v>
-      </c>
-      <c r="G51" s="1" t="s">
-        <v>301</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="D52" s="1" t="s">
         <v>302</v>
       </c>
-      <c r="B52" s="2" t="s">
+      <c r="E52" s="1" t="s">
         <v>303</v>
       </c>
-      <c r="C52" s="1" t="s">
+      <c r="F52" s="1" t="s">
         <v>304</v>
       </c>
-      <c r="D52" s="1" t="s">
+      <c r="G52" s="1" t="s">
         <v>305</v>
-      </c>
-      <c r="E52" s="1" t="s">
-        <v>306</v>
-      </c>
-      <c r="F52" s="1" t="s">
-        <v>307</v>
-      </c>
-      <c r="G52" s="1" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="D53" s="1" t="s">
         <v>309</v>
       </c>
-      <c r="B53" s="2" t="s">
+      <c r="E53" s="1" t="s">
         <v>310</v>
       </c>
-      <c r="C53" s="1" t="s">
+      <c r="F53" s="1" t="s">
         <v>311</v>
       </c>
-      <c r="D53" s="1" t="s">
+      <c r="G53" s="1" t="s">
         <v>312</v>
-      </c>
-      <c r="E53" s="1" t="s">
-        <v>313</v>
-      </c>
-      <c r="F53" s="1" t="s">
-        <v>314</v>
-      </c>
-      <c r="G53" s="1" t="s">
-        <v>315</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="D54" s="1" t="s">
         <v>316</v>
       </c>
-      <c r="B54" s="2" t="n">
-        <v>300322</v>
-      </c>
-      <c r="C54" s="1" t="s">
+      <c r="E54" s="1" t="s">
         <v>317</v>
       </c>
-      <c r="D54" s="1" t="s">
+      <c r="F54" s="1" t="s">
         <v>318</v>
       </c>
-      <c r="E54" s="1" t="s">
+      <c r="G54" s="1" t="s">
         <v>319</v>
-      </c>
-      <c r="F54" s="1" t="s">
-        <v>320</v>
-      </c>
-      <c r="G54" s="1" t="s">
-        <v>321</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="B55" s="2" t="n">
+        <v>300322</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="D55" s="1" t="s">
         <v>322</v>
       </c>
-      <c r="B55" s="2" t="n">
-        <v>243500</v>
-      </c>
-      <c r="C55" s="1" t="s">
+      <c r="E55" s="1" t="s">
         <v>323</v>
       </c>
-      <c r="D55" s="1" t="s">
+      <c r="F55" s="1" t="s">
         <v>324</v>
       </c>
-      <c r="E55" s="1" t="s">
+      <c r="G55" s="1" t="s">
         <v>325</v>
-      </c>
-      <c r="F55" s="1" t="s">
-        <v>326</v>
-      </c>
-      <c r="G55" s="1" t="s">
-        <v>327</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="B56" s="2" t="n">
+        <v>243500</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="D56" s="1" t="s">
         <v>328</v>
       </c>
-      <c r="B56" s="2" t="n">
-        <v>609016</v>
-      </c>
-      <c r="C56" s="1" t="s">
+      <c r="E56" s="1" t="s">
         <v>329</v>
       </c>
-      <c r="D56" s="1" t="s">
+      <c r="F56" s="1" t="s">
         <v>330</v>
       </c>
-      <c r="E56" s="1" t="s">
+      <c r="G56" s="1" t="s">
         <v>331</v>
-      </c>
-      <c r="F56" s="1" t="s">
-        <v>332</v>
-      </c>
-      <c r="G56" s="1" t="s">
-        <v>333</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="B57" s="2" t="n">
+        <v>609016</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="D57" s="1" t="s">
         <v>334</v>
       </c>
-      <c r="B57" s="2" t="n">
-        <v>143450</v>
-      </c>
-      <c r="C57" s="1" t="s">
+      <c r="E57" s="1" t="s">
         <v>335</v>
       </c>
-      <c r="D57" s="1" t="s">
+      <c r="F57" s="1" t="s">
         <v>336</v>
       </c>
-      <c r="E57" s="1" t="s">
+      <c r="G57" s="1" t="s">
         <v>337</v>
-      </c>
-      <c r="F57" s="1" t="s">
-        <v>338</v>
-      </c>
-      <c r="G57" s="1" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="B58" s="2" t="n">
+        <v>143450</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="D58" s="1" t="s">
         <v>340</v>
       </c>
-      <c r="B58" s="2" t="n">
-        <v>222700</v>
-      </c>
-      <c r="C58" s="1" t="s">
+      <c r="E58" s="1" t="s">
         <v>341</v>
       </c>
-      <c r="D58" s="1" t="s">
+      <c r="F58" s="1" t="s">
         <v>342</v>
       </c>
-      <c r="E58" s="1" t="s">
+      <c r="G58" s="1" t="s">
         <v>343</v>
-      </c>
-      <c r="F58" s="1" t="s">
-        <v>344</v>
-      </c>
-      <c r="G58" s="1" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="B59" s="2" t="n">
+        <v>222700</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="D59" s="1" t="s">
         <v>346</v>
       </c>
-      <c r="B59" s="2" t="n">
-        <v>248360</v>
-      </c>
-      <c r="C59" s="1" t="s">
+      <c r="E59" s="1" t="s">
         <v>347</v>
       </c>
-      <c r="D59" s="1" t="s">
+      <c r="F59" s="1" t="s">
         <v>348</v>
       </c>
-      <c r="E59" s="1" t="s">
+      <c r="G59" s="1" t="s">
         <v>349</v>
-      </c>
-      <c r="F59" s="1" t="s">
-        <v>350</v>
-      </c>
-      <c r="G59" s="1" t="s">
-        <v>351</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="B60" s="2" t="n">
+        <v>248360</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="D60" s="1" t="s">
         <v>352</v>
       </c>
-      <c r="B60" s="2" t="n">
-        <v>248600</v>
-      </c>
-      <c r="C60" s="1" t="s">
+      <c r="E60" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D60" s="1" t="s">
+      <c r="F60" s="1" t="s">
         <v>354</v>
       </c>
-      <c r="E60" s="1" t="s">
+      <c r="G60" s="1" t="s">
         <v>355</v>
-      </c>
-      <c r="F60" s="1" t="s">
-        <v>356</v>
-      </c>
-      <c r="G60" s="1" t="s">
-        <v>357</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="B61" s="2" t="n">
+        <v>248600</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>357</v>
+      </c>
+      <c r="D61" s="1" t="s">
         <v>358</v>
       </c>
-      <c r="B61" s="2" t="n">
-        <v>201450</v>
-      </c>
-      <c r="C61" s="1" t="s">
+      <c r="E61" s="1" t="s">
         <v>359</v>
       </c>
-      <c r="D61" s="1" t="s">
+      <c r="F61" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="E61" s="1" t="s">
+      <c r="G61" s="1" t="s">
         <v>361</v>
-      </c>
-      <c r="F61" s="1" t="s">
-        <v>362</v>
-      </c>
-      <c r="G61" s="1" t="s">
-        <v>363</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="B62" s="2" t="n">
+        <v>201450</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="D62" s="1" t="s">
         <v>364</v>
       </c>
-      <c r="B62" s="2" t="n">
-        <v>250850</v>
-      </c>
-      <c r="C62" s="1" t="s">
+      <c r="E62" s="1" t="s">
         <v>365</v>
       </c>
-      <c r="D62" s="1" t="s">
+      <c r="F62" s="1" t="s">
         <v>366</v>
       </c>
-      <c r="E62" s="1" t="s">
+      <c r="G62" s="1" t="s">
         <v>367</v>
-      </c>
-      <c r="F62" s="1" t="s">
-        <v>368</v>
-      </c>
-      <c r="G62" s="1" t="s">
-        <v>369</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="B63" s="2" t="n">
+        <v>250850</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="D63" s="1" t="s">
         <v>370</v>
       </c>
-      <c r="B63" s="2" t="n">
-        <v>251000</v>
-      </c>
-      <c r="C63" s="1" t="s">
+      <c r="E63" s="1" t="s">
         <v>371</v>
       </c>
-      <c r="D63" s="1" t="s">
+      <c r="F63" s="1" t="s">
         <v>372</v>
       </c>
-      <c r="E63" s="1" t="s">
+      <c r="G63" s="1" t="s">
         <v>373</v>
-      </c>
-      <c r="F63" s="1" t="s">
-        <v>374</v>
-      </c>
-      <c r="G63" s="1" t="s">
-        <v>375</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
+        <v>374</v>
+      </c>
+      <c r="B64" s="2" t="n">
+        <v>251000</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="D64" s="1" t="s">
         <v>376</v>
       </c>
-      <c r="B64" s="2" t="n">
-        <v>251120</v>
-      </c>
-      <c r="C64" s="1" t="s">
+      <c r="E64" s="1" t="s">
         <v>377</v>
       </c>
-      <c r="D64" s="1" t="s">
+      <c r="F64" s="1" t="s">
         <v>378</v>
-      </c>
-      <c r="E64" s="1" t="s">
-        <v>36</v>
       </c>
       <c r="G64" s="1" t="s">
         <v>379</v>
@@ -3354,7 +3356,7 @@
         <v>380</v>
       </c>
       <c r="B65" s="2" t="n">
-        <v>260920</v>
+        <v>251120</v>
       </c>
       <c r="C65" s="1" t="s">
         <v>381</v>
@@ -3363,41 +3365,41 @@
         <v>382</v>
       </c>
       <c r="E65" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G65" s="1" t="s">
         <v>383</v>
-      </c>
-      <c r="F65" s="1" t="s">
-        <v>384</v>
-      </c>
-      <c r="G65" s="1" t="s">
-        <v>385</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="B66" s="2" t="n">
+        <v>260920</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>385</v>
+      </c>
+      <c r="D66" s="1" t="s">
         <v>386</v>
       </c>
-      <c r="B66" s="2" t="s">
+      <c r="E66" s="1" t="s">
         <v>387</v>
       </c>
-      <c r="C66" s="1" t="s">
+      <c r="F66" s="1" t="s">
         <v>388</v>
       </c>
-      <c r="D66" s="1" t="s">
+      <c r="G66" s="1" t="s">
         <v>389</v>
-      </c>
-      <c r="E66" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="G66" s="1" t="s">
-        <v>390</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="B67" s="2" t="s">
         <v>391</v>
-      </c>
-      <c r="B67" s="2" t="n">
-        <v>252450</v>
       </c>
       <c r="C67" s="1" t="s">
         <v>392</v>
@@ -3406,30 +3408,30 @@
         <v>393</v>
       </c>
       <c r="E67" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G67" s="1" t="s">
         <v>394</v>
-      </c>
-      <c r="F67" s="1" t="s">
-        <v>395</v>
-      </c>
-      <c r="G67" s="1" t="s">
-        <v>396</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="B68" s="2" t="n">
+        <v>252450</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="D68" s="1" t="s">
         <v>397</v>
       </c>
-      <c r="B68" s="2" t="n">
-        <v>611412</v>
-      </c>
-      <c r="C68" s="1" t="s">
+      <c r="E68" s="1" t="s">
         <v>398</v>
       </c>
-      <c r="D68" s="1" t="s">
+      <c r="F68" s="1" t="s">
         <v>399</v>
-      </c>
-      <c r="E68" s="1" t="s">
-        <v>36</v>
       </c>
       <c r="G68" s="1" t="s">
         <v>400</v>
@@ -3439,221 +3441,221 @@
       <c r="A69" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="B69" s="2" t="s">
+      <c r="B69" s="2" t="n">
+        <v>611412</v>
+      </c>
+      <c r="C69" s="1" t="s">
         <v>402</v>
       </c>
-      <c r="C69" s="1" t="s">
+      <c r="D69" s="1" t="s">
         <v>403</v>
-      </c>
-      <c r="D69" s="1" t="s">
-        <v>404</v>
       </c>
       <c r="E69" s="1" t="s">
         <v>36</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="1" t="s">
+        <v>405</v>
+      </c>
+      <c r="B70" s="2" t="s">
         <v>406</v>
       </c>
-      <c r="B70" s="2" t="s">
+      <c r="C70" s="1" t="s">
         <v>407</v>
       </c>
-      <c r="C70" s="1" t="s">
+      <c r="D70" s="1" t="s">
         <v>408</v>
       </c>
-      <c r="D70" s="1" t="s">
+      <c r="E70" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G70" s="1" t="s">
         <v>409</v>
-      </c>
-      <c r="E70" s="1" t="s">
-        <v>410</v>
-      </c>
-      <c r="F70" s="1" t="s">
-        <v>411</v>
-      </c>
-      <c r="G70" s="1" t="s">
-        <v>412</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="D71" s="1" t="s">
         <v>413</v>
       </c>
-      <c r="B71" s="2" t="n">
+      <c r="E71" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="F71" s="1" t="s">
+        <v>415</v>
+      </c>
+      <c r="G71" s="1" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="B72" s="2" t="n">
         <v>258870</v>
       </c>
-      <c r="C71" s="1" t="s">
-        <v>414</v>
-      </c>
-      <c r="D71" s="1" t="s">
-        <v>415</v>
-      </c>
-      <c r="E71" s="1" t="s">
-        <v>416</v>
-      </c>
-      <c r="F71" s="1" t="s">
-        <v>417</v>
-      </c>
-      <c r="G71" s="1" t="s">
+      <c r="C72" s="1" t="s">
         <v>418</v>
       </c>
-    </row>
-    <row r="72" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="1" t="s">
+      <c r="D72" s="1" t="s">
         <v>419</v>
       </c>
-      <c r="B72" s="2" t="n">
+      <c r="E72" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="F72" s="1" t="s">
+        <v>421</v>
+      </c>
+      <c r="G72" s="1" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A73" s="1" t="s">
+        <v>423</v>
+      </c>
+      <c r="B73" s="2" t="n">
         <v>311250</v>
       </c>
-      <c r="C72" s="1" t="s">
-        <v>420</v>
-      </c>
-      <c r="D72" s="1" t="s">
-        <v>421</v>
-      </c>
-      <c r="E72" s="1" t="s">
-        <v>422</v>
-      </c>
-      <c r="F72" s="1" t="s">
-        <v>423</v>
-      </c>
-      <c r="G72" s="1" t="s">
+      <c r="C73" s="1" t="s">
         <v>424</v>
       </c>
-    </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="1" t="s">
+      <c r="D73" s="1" t="s">
         <v>425</v>
       </c>
-      <c r="B73" s="2" t="n">
+      <c r="E73" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="F73" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="G73" s="1" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A74" s="1" t="s">
+        <v>429</v>
+      </c>
+      <c r="B74" s="2" t="n">
         <v>261600</v>
       </c>
-      <c r="C73" s="1" t="s">
-        <v>426</v>
-      </c>
-      <c r="D73" s="1" t="s">
-        <v>427</v>
-      </c>
-      <c r="E73" s="1" t="s">
-        <v>428</v>
-      </c>
-      <c r="F73" s="1" t="s">
-        <v>429</v>
-      </c>
-      <c r="G73" s="1" t="s">
+      <c r="C74" s="1" t="s">
         <v>430</v>
       </c>
-    </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="1" t="s">
+      <c r="D74" s="1" t="s">
         <v>431</v>
       </c>
-      <c r="B74" s="2" t="n">
-        <v>170100</v>
-      </c>
-      <c r="C74" s="1" t="s">
+      <c r="E74" s="1" t="s">
         <v>432</v>
       </c>
-      <c r="D74" s="1" t="s">
+      <c r="F74" s="1" t="s">
         <v>433</v>
       </c>
-      <c r="E74" s="1" t="s">
+      <c r="G74" s="1" t="s">
         <v>434</v>
-      </c>
-      <c r="F74" s="1" t="s">
-        <v>435</v>
-      </c>
-      <c r="G74" s="1" t="s">
-        <v>436</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="1" t="s">
+        <v>435</v>
+      </c>
+      <c r="B75" s="2" t="n">
+        <v>170100</v>
+      </c>
+      <c r="C75" s="1" t="s">
+        <v>436</v>
+      </c>
+      <c r="D75" s="1" t="s">
         <v>437</v>
       </c>
-      <c r="B75" s="2" t="s">
+      <c r="E75" s="1" t="s">
         <v>438</v>
       </c>
-      <c r="C75" s="1" t="s">
+      <c r="F75" s="1" t="s">
         <v>439</v>
       </c>
-      <c r="D75" s="1" t="s">
+      <c r="G75" s="1" t="s">
         <v>440</v>
-      </c>
-      <c r="E75" s="1" t="s">
-        <v>441</v>
-      </c>
-      <c r="F75" s="1" t="s">
-        <v>442</v>
-      </c>
-      <c r="G75" s="1" t="s">
-        <v>443</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="1" t="s">
+        <v>441</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="D76" s="1" t="s">
         <v>444</v>
       </c>
-      <c r="B76" s="2" t="n">
-        <v>606054</v>
-      </c>
-      <c r="C76" s="1" t="s">
+      <c r="E76" s="1" t="s">
         <v>445</v>
       </c>
-      <c r="D76" s="1" t="s">
+      <c r="F76" s="1" t="s">
         <v>446</v>
       </c>
-      <c r="E76" s="1" t="s">
+      <c r="G76" s="1" t="s">
         <v>447</v>
-      </c>
-      <c r="F76" s="1" t="s">
-        <v>448</v>
-      </c>
-      <c r="G76" s="1" t="s">
-        <v>449</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="1" t="s">
+        <v>448</v>
+      </c>
+      <c r="B77" s="2" t="n">
+        <v>606054</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>449</v>
+      </c>
+      <c r="D77" s="1" t="s">
         <v>450</v>
       </c>
-      <c r="B77" s="2" t="n">
-        <v>266500</v>
-      </c>
-      <c r="C77" s="1" t="s">
+      <c r="E77" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="D77" s="1" t="s">
+      <c r="F77" s="1" t="s">
         <v>452</v>
       </c>
-      <c r="E77" s="1" t="s">
+      <c r="G77" s="1" t="s">
         <v>453</v>
-      </c>
-      <c r="F77" s="1" t="s">
-        <v>454</v>
-      </c>
-      <c r="G77" s="1" t="s">
-        <v>455</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="B78" s="2" t="n">
+        <v>266500</v>
+      </c>
+      <c r="C78" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="D78" s="1" t="s">
         <v>456</v>
       </c>
-      <c r="B78" s="2" t="n">
-        <v>614707</v>
-      </c>
-      <c r="C78" s="1" t="s">
+      <c r="E78" s="1" t="s">
         <v>457</v>
       </c>
-      <c r="D78" s="1" t="s">
+      <c r="F78" s="1" t="s">
         <v>458</v>
-      </c>
-      <c r="E78" s="1" t="s">
-        <v>36</v>
       </c>
       <c r="G78" s="1" t="s">
         <v>459</v>
@@ -3663,51 +3665,51 @@
       <c r="A79" s="1" t="s">
         <v>460</v>
       </c>
-      <c r="B79" s="2" t="s">
+      <c r="B79" s="2" t="n">
+        <v>614707</v>
+      </c>
+      <c r="C79" s="1" t="s">
         <v>461</v>
       </c>
-      <c r="C79" s="1" t="s">
+      <c r="D79" s="1" t="s">
         <v>462</v>
       </c>
-      <c r="D79" s="1" t="s">
+      <c r="E79" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G79" s="1" t="s">
         <v>463</v>
-      </c>
-      <c r="E79" s="1" t="s">
-        <v>464</v>
-      </c>
-      <c r="F79" s="1" t="s">
-        <v>465</v>
-      </c>
-      <c r="G79" s="1" t="s">
-        <v>466</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="1" t="s">
+        <v>464</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>465</v>
+      </c>
+      <c r="C80" s="1" t="s">
+        <v>466</v>
+      </c>
+      <c r="D80" s="1" t="s">
         <v>467</v>
       </c>
-      <c r="B80" s="2" t="s">
+      <c r="E80" s="1" t="s">
         <v>468</v>
       </c>
-      <c r="C80" s="1" t="s">
+      <c r="F80" s="1" t="s">
         <v>469</v>
       </c>
-      <c r="D80" s="1" t="s">
+      <c r="G80" s="1" t="s">
         <v>470</v>
-      </c>
-      <c r="E80" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="G80" s="1" t="s">
-        <v>471</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="B81" s="2" t="s">
         <v>472</v>
-      </c>
-      <c r="B81" s="2" t="n">
-        <v>201470</v>
       </c>
       <c r="C81" s="1" t="s">
         <v>473</v>
@@ -3716,53 +3718,53 @@
         <v>474</v>
       </c>
       <c r="E81" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G81" s="1" t="s">
         <v>475</v>
-      </c>
-      <c r="F81" s="1" t="s">
-        <v>476</v>
-      </c>
-      <c r="G81" s="1" t="s">
-        <v>477</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="B82" s="2" t="n">
+        <v>201470</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>477</v>
+      </c>
+      <c r="D82" s="1" t="s">
         <v>478</v>
       </c>
-      <c r="B82" s="2" t="n">
-        <v>600737</v>
-      </c>
-      <c r="C82" s="1" t="s">
+      <c r="E82" s="1" t="s">
         <v>479</v>
       </c>
-      <c r="D82" s="1" t="s">
+      <c r="F82" s="1" t="s">
         <v>480</v>
       </c>
-      <c r="E82" s="1" t="s">
+      <c r="G82" s="1" t="s">
         <v>481</v>
-      </c>
-      <c r="F82" s="1" t="s">
-        <v>482</v>
-      </c>
-      <c r="G82" s="1" t="s">
-        <v>483</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="B83" s="2" t="n">
+        <v>600737</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>483</v>
+      </c>
+      <c r="D83" s="1" t="s">
         <v>484</v>
       </c>
-      <c r="B83" s="2" t="n">
-        <v>212140</v>
-      </c>
-      <c r="C83" s="1" t="s">
+      <c r="E83" s="1" t="s">
         <v>485</v>
       </c>
-      <c r="D83" s="1" t="s">
+      <c r="F83" s="1" t="s">
         <v>486</v>
-      </c>
-      <c r="E83" s="1" t="s">
-        <v>36</v>
       </c>
       <c r="G83" s="1" t="s">
         <v>487</v>
@@ -3773,7 +3775,7 @@
         <v>488</v>
       </c>
       <c r="B84" s="2" t="n">
-        <v>184420</v>
+        <v>212140</v>
       </c>
       <c r="C84" s="1" t="s">
         <v>489</v>
@@ -3793,7 +3795,7 @@
         <v>492</v>
       </c>
       <c r="B85" s="2" t="n">
-        <v>271980</v>
+        <v>184420</v>
       </c>
       <c r="C85" s="1" t="s">
         <v>493</v>
@@ -3802,53 +3804,53 @@
         <v>494</v>
       </c>
       <c r="E85" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G85" s="1" t="s">
         <v>495</v>
-      </c>
-      <c r="F85" s="1" t="s">
-        <v>496</v>
-      </c>
-      <c r="G85" s="1" t="s">
-        <v>497</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="B86" s="2" t="n">
+        <v>271980</v>
+      </c>
+      <c r="C86" s="1" t="s">
+        <v>497</v>
+      </c>
+      <c r="D86" s="1" t="s">
         <v>498</v>
       </c>
-      <c r="B86" s="2" t="n">
-        <v>606003</v>
-      </c>
-      <c r="C86" s="1" t="s">
+      <c r="E86" s="1" t="s">
         <v>499</v>
       </c>
-      <c r="D86" s="1" t="s">
+      <c r="F86" s="1" t="s">
         <v>500</v>
       </c>
-      <c r="E86" s="1" t="s">
+      <c r="G86" s="1" t="s">
         <v>501</v>
-      </c>
-      <c r="F86" s="1" t="s">
-        <v>502</v>
-      </c>
-      <c r="G86" s="1" t="s">
-        <v>503</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="B87" s="2" t="n">
+        <v>606003</v>
+      </c>
+      <c r="C87" s="1" t="s">
+        <v>503</v>
+      </c>
+      <c r="D87" s="1" t="s">
         <v>504</v>
       </c>
-      <c r="B87" s="2" t="n">
-        <v>300872</v>
-      </c>
-      <c r="C87" s="1" t="s">
+      <c r="E87" s="1" t="s">
         <v>505</v>
       </c>
-      <c r="D87" s="1" t="s">
+      <c r="F87" s="1" t="s">
         <v>506</v>
-      </c>
-      <c r="E87" s="1" t="s">
-        <v>36</v>
       </c>
       <c r="G87" s="1" t="s">
         <v>507</v>
@@ -3859,7 +3861,7 @@
         <v>508</v>
       </c>
       <c r="B88" s="2" t="n">
-        <v>276700</v>
+        <v>300872</v>
       </c>
       <c r="C88" s="1" t="s">
         <v>509</v>
@@ -3868,124 +3870,144 @@
         <v>510</v>
       </c>
       <c r="E88" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G88" s="1" t="s">
         <v>511</v>
-      </c>
-      <c r="F88" s="1" t="s">
-        <v>512</v>
-      </c>
-      <c r="G88" s="1" t="s">
-        <v>513</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="1" t="s">
+        <v>512</v>
+      </c>
+      <c r="B89" s="2" t="n">
+        <v>276700</v>
+      </c>
+      <c r="C89" s="1" t="s">
+        <v>513</v>
+      </c>
+      <c r="D89" s="1" t="s">
         <v>514</v>
       </c>
-      <c r="B89" s="2" t="n">
-        <v>258900</v>
-      </c>
-      <c r="C89" s="1" t="s">
+      <c r="E89" s="1" t="s">
         <v>515</v>
       </c>
-      <c r="D89" s="1" t="s">
+      <c r="F89" s="1" t="s">
         <v>516</v>
       </c>
-      <c r="E89" s="1" t="s">
+      <c r="G89" s="1" t="s">
         <v>517</v>
-      </c>
-      <c r="F89" s="1" t="s">
-        <v>518</v>
-      </c>
-      <c r="G89" s="1" t="s">
-        <v>519</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="1" t="s">
+        <v>518</v>
+      </c>
+      <c r="B90" s="2" t="n">
+        <v>258900</v>
+      </c>
+      <c r="C90" s="1" t="s">
+        <v>519</v>
+      </c>
+      <c r="D90" s="1" t="s">
         <v>520</v>
       </c>
-      <c r="B90" s="2" t="n">
-        <v>201475</v>
-      </c>
-      <c r="C90" s="1" t="s">
+      <c r="E90" s="1" t="s">
         <v>521</v>
       </c>
-      <c r="D90" s="1" t="s">
+      <c r="F90" s="1" t="s">
         <v>522</v>
       </c>
-      <c r="E90" s="1" t="s">
+      <c r="G90" s="1" t="s">
         <v>523</v>
-      </c>
-      <c r="F90" s="1" t="s">
-        <v>524</v>
-      </c>
-      <c r="G90" s="1" t="s">
-        <v>525</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="1" t="s">
+        <v>524</v>
+      </c>
+      <c r="B91" s="2" t="n">
+        <v>201475</v>
+      </c>
+      <c r="C91" s="1" t="s">
+        <v>525</v>
+      </c>
+      <c r="D91" s="1" t="s">
         <v>526</v>
       </c>
-      <c r="B91" s="2" t="n">
+      <c r="E91" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="F91" s="1" t="s">
+        <v>528</v>
+      </c>
+      <c r="G91" s="1" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="1" t="s">
+        <v>530</v>
+      </c>
+      <c r="B92" s="2" t="n">
         <v>603592</v>
       </c>
-      <c r="C91" s="1" t="s">
-        <v>527</v>
-      </c>
-      <c r="D91" s="1" t="s">
-        <v>528</v>
-      </c>
-      <c r="E91" s="1" t="s">
-        <v>529</v>
-      </c>
-      <c r="F91" s="1" t="s">
-        <v>530</v>
-      </c>
-      <c r="G91" s="1" t="s">
+      <c r="C92" s="1" t="s">
         <v>531</v>
       </c>
-    </row>
-    <row r="92" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A92" s="1" t="s">
+      <c r="D92" s="1" t="s">
         <v>532</v>
       </c>
-      <c r="B92" s="2" t="n">
+      <c r="E92" s="1" t="s">
+        <v>533</v>
+      </c>
+      <c r="F92" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="G92" s="1" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A93" s="1" t="s">
+        <v>536</v>
+      </c>
+      <c r="B93" s="2" t="n">
         <v>234580</v>
       </c>
-      <c r="C92" s="1" t="s">
-        <v>533</v>
-      </c>
-      <c r="D92" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="E92" s="1" t="s">
-        <v>535</v>
-      </c>
-      <c r="F92" s="1" t="s">
-        <v>536</v>
-      </c>
-      <c r="G92" s="1" t="s">
+      <c r="C93" s="1" t="s">
         <v>537</v>
       </c>
-    </row>
-    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="1" t="s">
+      <c r="D93" s="1" t="s">
         <v>538</v>
+      </c>
+      <c r="E93" s="1" t="s">
+        <v>539</v>
+      </c>
+      <c r="F93" s="1" t="s">
+        <v>540</v>
+      </c>
+      <c r="G93" s="1" t="s">
+        <v>541</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="1" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="1" t="s">
-        <v>540</v>
+        <v>543</v>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="1" t="s">
+        <v>544</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D90"/>
+  <autoFilter ref="A1:D91"/>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" display="236792; 600721"/>
   </hyperlinks>

</xml_diff>

<commit_message>
Changed some biomarkers in the excel
</commit_message>
<xml_diff>
--- a/pathway_pipeline/iembase-diseases-with-pathbank-pathways-and-hmdb-codes.xlsx
+++ b/pathway_pipeline/iembase-diseases-with-pathbank-pathways-and-hmdb-codes.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="544">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="543">
   <si>
     <t xml:space="preserve">Disease</t>
   </si>
@@ -515,6 +515,39 @@
   </si>
   <si>
     <t xml:space="preserve">BCKDK </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Isoleucine ↓; Leucine ↓; Valine ↓; alpha-Ketoisovaleric acid ↓; 3-Methyl-2-oxovaleric acid ↓</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Isoleucine (HMDB0000172); Leucine (HMDB0000687); Valine (HMDB0000883); alpha-Ketoisovaleric acid (HMDB0000019); 3-Methyl-2-oxovaleric acid (HMDB0000491)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Canavan disease</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N-Acetylaspartic acid ↑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Canavan Disease (PathBank PW000093)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMP0000175</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N-Acetyl-L-aspartic acid (HMDB0000812)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carbamoyl-phosphate synthetase I deficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">237300 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPS1 </t>
   </si>
   <si>
     <r>
@@ -525,7 +558,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">Isoleucine ↓; Leucine ↓; Valine ↓; alpha-Ketoisovaleric acid </t>
+      <t xml:space="preserve">Arginine ↓; Citrulline ↓; Glutamine </t>
     </r>
     <r>
       <rPr>
@@ -534,43 +567,10 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">↓; 3-Methyl-2-oxovaleric acid ↓</t>
+      <t xml:space="preserve">↑</t>
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Isoleucine (HMDB0000172); Leucine (HMDB0000687); Valine (HMDB0000883); alpha-Ketoisovaleric acid (HMDB0000019); 3-Methyl-2-oxovaleric acid (HMDB0000491)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Canavan disease</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N-Acetylaspartic acid ↑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Canavan Disease (PathBank PW000093)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMP0000175</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N-Acetyl-L-aspartic acid (HMDB0000812)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Carbamoyl-phosphate synthetase I deficiency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">237300 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPS1 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arginine ↓; Citrulline ↓; Glutamine ↓</t>
-  </si>
-  <si>
     <t xml:space="preserve">Carbamoyl Phosphate Synthetase Deficiency (PathBank PW000191)</t>
   </si>
   <si>
@@ -602,669 +602,6 @@
   </si>
   <si>
     <t xml:space="preserve">CTLN2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Citrulline ↑; Arginine ↑; Glutamine ↑; Threonine ↑; Thr/Ser ↑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arginine (HMDB0000517); Citrulline (HMDB0000904); Glutamine (HMDB0000641); Threonine (HMDB0000167)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Citrullinemia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CTLN1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Citrulline ↑; N-Acetylcitrulline ↑; Arginine ↓</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Citrullinemia Type I (PathBank PW000185)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMP0000001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Citrulline (HMDB0000904); N-Acetylcitrulline (HMDB0000856); Arginine (HMDB0000517)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPT1A deficiency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPT1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-carnitine ↑; Palmitoylcarnitine ↓; Stearoylcarnitine ↓;  C0/(C16+C18) ↑ </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Carnitine Palmitoyl Transferase Deficiency I (PathBank PW</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMP0125739</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-Carnitine (HMDB0000062); Palmitoylcarnitine (HMDB0000222); Stearoylcarnitine (HMDB0000848)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPT2 deficiency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPT2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-carnitine ↓; Palmitoylcarnitine ↑; Oleoylcarnitine ↑; (C16+C18:1)/C2 ↑ </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Carnitine Palmitoyl Transferase Deficiency II </t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMP0658967</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-Carnitine (HMDB0000062); Palmitoylcarnitine (HMDB0000222); Oleoylcarnitine (HMDB0005065)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cystathionine beta-synthase deficiency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBS </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Methionine ↑; Glutamyl-methionine ↑; Methionine-hexose ↑; 5'-Methylthioadenosine ↑; Homocysteine ↑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cystathionine beta-Synthase Deficiency (PathBank PW000100)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMP0000177</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Methionine (HMDB0000696); Glutamyl-methionine (HMDB0034367); Methionine-hexose (no HMDB entry found); 5'-Methylthioadenosine (HMDB0001173); Homocysteine (HMDB0000742)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cytosolic phosphoenolpyruvate carboxykinase deficiency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">261680 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">PEPCK-C </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Glutamine ↑; Arginine ↓; Citrulline ↓ </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Phosphoenolpyruvate Carboxykinase Deficiency 1 (PEPCK1) (PathBank PW000536)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMP0000560</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Glutamine (HMDB0000641); Arginine (HMDB0000517); Citrulline (HMDB0000904)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dihydropyrimidinase deficiency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DPH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dihydrothymine ↑; Dihydrouracil ↑; Thymine ↑; Uracil ↑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dihydropyrimidinase Deficiency (PathBank PW000189)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMP0000178</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dihydrothymine (HMDB0000079); Dihydrouracil (HMDB0000076); Thymine (HMDB0000262); Uracil (HMDB0000300)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dihydropyrimidine dehydrogenase deficiency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DPD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thymine ↑; Uracil ↑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dihydropyrimidine Dehydrogenase Deficiency (DHPD) (PathBank PW000198)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMP0000179</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thymine (HMDB0000262); Uracil (HMDB0000300)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dimethylglycine dehydrogenase deficiency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">605849 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">DMGLY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dimethylglycine ↑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dimethylglycine Dehydrogenase Deficiency (PathBank PW000197)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMP0000242</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dimethylglycine (HMDB0000092)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DNAJC12 deficiency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">606060 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">DNAJC12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Phenylalanine ↑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Phenylalanine (HMDB0000159)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ethylmalonic encephalopathy (ETHE1 deficiency)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">602473 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">ETHE1 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ethylmalonic acid ↑; 2-Methylbutyrylglycine ↑; Methylsuccinic acid ↑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ethylmalonic Encephalopathy (PathBank PW000106)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMP0000181</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ethylmalonic acid (HMDB0000622); 2-Methylbutyrylglycine (HMDB0000339); Methylsuccinic acid (HMDB0001844)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Formimidoyltransferase cyclodeaminase deficiency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">229100 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">FIGLU </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hydantoin-5-propionic acid ↑; Formiminoglutamic acid ↑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hydantoin-5-propionic acid (HMDB0001212); Formiminoglutamic acid (HMDB0000854)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fumarate hydratase deficiency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">606812 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">FH1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fumaric acid ↑; Succinic acid ↑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fumarase Deficiency (PathBank PW000523)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMP0000547</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fumaric acid (HMDB0000134); Succinic acid (HMDB0000254)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Galactosemia type 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">230400 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">GAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Galactose ↑; Galactitol ↑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Galactosemia (PathBank PW000200)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMP0000182</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Galactose (HMDB0000143); Galactitol (HMDB0000107)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Glucose transporter 1 deficiency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GLUT1-D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Glucose ↓*; Gluconic + Galactonic acid ↓*; Xylose-α1-3-glucose ↓*; Xylose-α1-3-xylose-α1-3-glucose↓*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GLUT-1 Deficiency Syndrome (PathBank PW000556)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMP0000580</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Glucose (HMDB0000122); Gluconic + Galactonic acid (HMDB0000625; HMDB0000565); Xylose-α1-3-glucose (no HMDB entry found); Xylose-α1-3-xylose-α1-3-glucose (no HMDB entry found)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Glucose transporter 2 deficiency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">227810 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">FBS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fanconi-Bickel Syndrome (PathBank PW000548)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMP0000572</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Glutaric aciduria type II</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GA2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Glutaric acid ↑; Glutarylcarnitine ↑; 3-Hydroxyglutaric acid ↑; Hexanoylcarnitine ↑; Octanoylcarnitine ↑; 3, 5-Tetradecadiencarnitine ↑; cis-5-Tetradecenoylcarnitine ↑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Glutaric acid (HMDB0000661); Glutarylcarnitine (HMDB0013130); 3-Hydroxyglutaric acid (HMDB0000428); Hexanoylcarnitine (HMDB0000756); Octanoylcarnitine (HMDB0000791); 3, 5-Tetradecadiencarnitine (HMDB0241375); cis-5-Tetradecenoylcarnitine (HMDB0002014)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Glutaryl-CoA dehydrogenase deficiency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">231670 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">GA-1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Glutaric acid ↑; Glutarylcarnitine ↑; 3-Hydroxyglutaric acid ↑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Glutaric Aciduria Type I (PathBank PW000107)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMP0000185</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Glutaric acid (HMDB0000661); Glutarylcarnitine (HMDB0013130); 3-Hydroxyglutaric acid (HMDB0000428)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Guanidinoacetate methyltransferase deficiency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">612736 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">GAMT </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Guanidinoacetic acid ↑; Creatine ↓; Creatinine ↓</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Guanidinoacetate Methyltransferase Deficiency (GAMT Deficiency) (PathBank PW000088)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMP0000188</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Guanidinoacetic acid (HMDB0000128); Creatine (HMDB0000064); Creatinine (HMDB0000562)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Histidine ammonia-lyase deficiency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">235800 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">HAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Histidine ↑; Imidazole lactic acid ↑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Histidinemia (PathBank PW000113)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMP0000191</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Histidine (HMDB0000177); Imidazole lactic acid (HMDB0002320)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Homogentisic acid oxidase deficiency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">203500 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">AKU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Homogentisic acid ↑; Tyrosine ↑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alkaptonuria (PathBank PW000180)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMP0000169</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Homogentisic acid (not observed in our plasma data) (HMDB0000130); Tyrosine (HMDB0000158)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hyperprolinemia type 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">239510 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">P5CDH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Proline ↑; Pyrrole-2-carboxylic acid ↑; 2-Pyrroloylglycine ↑; Pyrrole-2-carboxylic acid ↑; (2 R)-5-(2-oxopropyl)pyrrolidine-2-carboxylic acid ↑; (2 R)-5-(carboxymethyl)pyrrolidine-2-carboxylic acid ↑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hyperprolinemia Type II (PathBank PW000085)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMP0000360</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Proline (HMDB0000162); Pyrrole-2-carboxylic acid (HMDB0004230); 2-Pyrroloylglycine (HMDB0059778); Pyrrole-2-carboxylic acid (HMDB0004230); (2 R)-5-(2-oxopropyl)pyrrolidine-2-carboxylic acid (no HMDB entry found); (2 R)-5-(carboxymethyl)pyrrolidine-2-carboxylic acid (no HMDB entry found)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hypoxanthine guanine phosphoribosyltransferase deficiency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HGPRT </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hypoxanthine ↑; Xanthine ↑; Uric acid ↑; AICA riboside ↑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lesch-Nyhan Syndrome (LNS) (PathBank PW000078)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMP0000364</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hypoxanthine (HMDB0000157); Xanthine (HMDB0000292); Uric acid (HMDB0000289); AICA riboside (HMDB0062179)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Isovaleryl-CoA dehydrogenase deficiency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IVA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Isovalerylglycine ↑; Isovalerylcarnitine ↑; Isovaleric acid ↑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Isovaleric Aciduria (PathBank PW000091)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMP0000238</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Isovalerylglycine (HMDB0000678); Isovalerylcarnitine (HMDB0000688); Isovaleric acid (HMDB0000718)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Long-chain 3-hydroxyacyl-CoA dehydrogenase deficiency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LCHAD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3-Hydroxyhexadecanoylcarnitine ↑; 3-Hydroxytetradecanoylcarnitine ↑;  3-Hydroxytetradecenoylcarnitine ↑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Long-Chain-3-Hydroxyacyl-CoA Dehydrogenase Deficiency (LCHAD) (PathBank PW000520)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMP0000544</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3-Hydroxyhexadecanoylcarnitine (HMDB0013336); 3-Hydroxytetradecanoylcarnitine (HMDB0061640); 3-Hydroxytetradecenoylcarnitine (HMDB0013330)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Long-chain 3-ketoacyl CoA thiolase deficiency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LCKAT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hexadecanoylcarnitine ↑; 3-Hydroxyhexadecanoylcarnitine ↑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trifunctional Protein Deficiency (PathBank PW000521)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMP0000545</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hexadecanoylcarnitine (HMDB0000222); 3-Hydroxyhexadecanoylcarnitine (HMDB0013336)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lysinuric protein intolerance (LPI)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LPI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lysine ↓; Arginine ↓; Ornithine ↓; Glutamine ↑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lysinuric Protein Intolerance (LPI) (PathBank PW000561)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMP0000585</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lysine (HMDB0000182); Arginine (HMDB0000517); Ornithine (HMDB0000214); Glutamine (HMDB0000641)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Malonyl-CoA decarboxylase deficiency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Malonylcarnitine ↑; Malonic acid ↑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Malonyl-CoA Decarboxylase Deficiency (PathBank PW000478)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMP0000502</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Malonylcarnitine (HMDB0002095); Malonic acid (HMDB0000691)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maple syrup urine disease</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MSUD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Leucine ↑; Isoleucine ↑; Ketoleucine ↑; 2-Hydroxy-3-methylbutyric acid ↑; 2-Ketoisovaleric acid ↑; 3-Methyl-2-oxovaleric acid ↑; 2-Hydroxycaproic acid ↑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maple Syrup Urine Disease (PathBank PW000064)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMP0000199</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Leucine (HMDB0000687); Isoleucine (HMDB0000172); Ketoleucine (HMDB0000695); 2-Hydroxy-3-methylbutyric acid (HMDB0000407); 2-Ketoisovaleric acid (HMDB0000019); 3-Methyl-2-oxovaleric acid (HMDB0000491); 2-Hydroxycaproic acid (HMDB0001624)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Medium-chain acyl-CoA dehydrogenase deficiency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MCAD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-Octanoylcarnitine ↑; Hexanoylglycine ↑; Hexanoylcarnitine ↑; 9-Decenoylcarnitine ↑; 2-trans,4-cis-Decadienoylcarnitine ↑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Medium Chain Acyl-CoA Dehydrogenase Deficiency (MCAD) (PathBank PW000518)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMP0000542</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L-Octanoylcarnitine (HMDB0000791); Hexanoylglycine (HMDB0000701); Hexanoylcarnitine (HMDB0000756); 9-Decenoylcarnitine (HMDB0013205); 2-trans,4-cis-Decadienoylcarnitine (HMDB0013325)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Methionine adenosyltransferase I/III deficiency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MAT I/III </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Methionine ↑; Glutamyl-methionine ↑; Methionine-hexose ↑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Methionine Adenosyltransferase Deficiency (PathBank PW000105)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMP0000221</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Methionine (HMDB0000696); Glutamyl-methionine (HMDB0034367); Methionine-hexose (no HMDB entry found)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Methylmalonic aciduria</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MMA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Methylmalonic acid ↑; Methylmalonylcarnitine ↑; Propionylcarnitine ↑; Propionic acid ↑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Methylmalonic Aciduria (PathBank PW000069)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMP0000200</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Methylmalonic acid (HMDB0000202); Methylmalonylcarnitine (HMDB0013133); Propionylcarnitine (HMDB0000824); Propionic acid (HMDB0000237)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mevalonate kinase deficiency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HIDS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mevalonic acid ↑; Mevalonolactone ↑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mevalonic Aciduria (PathBank PW000486)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMP0000510</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mevalonic acid (HMDB0000227); Mevalonolactone (HMDB0006024)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mitochondrial short-chain enoyl-CoA hydratase 1 deficiency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">616277 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">ECHS1D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pyruvate ↑; 2,3-Dihydroxy-2-methylbutanoic acid ↑; S-(2-carboxypropyl)-Cysteamine ↑; S-(2-Carboxypropyl)-cysteine ↑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pyruvate (HMDB0000243); 2,3-Dihydroxy-2-methylbutanoic acid (HMDB0029576); S-(2-carboxypropyl)-Cysteamine (HMDB0002169); S-(2-Carboxypropyl)-cysteine (no HMDB entry found)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Molybdenum cofactor deficiency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MOCD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Xanthosine ↑; Xanthine ↑;  2,3,4,5-Tetrahydropiperidine-2-carboxylate (P6C) ↑; 4-Pyridoxic acid ↑; Uric acid ↓</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Molybdenum Cofactor Deficiency (PathBank PW000079)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMP0000203</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Xanthosine (HMDB0000299); Xanthine (HMDB0000292); 2,3,4,5-Tetrahydropiperidine-2-carboxylate (P6C) (no HMDB entry found); 4-Pyridoxic acid (HMDB0000017); Uric acid (HMDB0000289)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N-acetylneuraminate pyruvate lyase deficiency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NPL -CDG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N-Acetylneuraminate ↑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N-Acetylneuraminate (HMDB0000230)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N-acetylneuraminic acid synthase deficiency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">610442 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">NANS-CDG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N-Acetylmannosamine ↑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N-Acetylmannosamine (HMDB0001129)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N-trimethyllysine hydroxylase deficiency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTSX6</t>
   </si>
   <si>
     <r>
@@ -1275,7 +612,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">4-Trimethylammoniobutanoic acid </t>
+      <t xml:space="preserve">Citrulline ↑; Arginine ↑; Glutamine </t>
     </r>
     <r>
       <rPr>
@@ -1284,8 +621,681 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">↓; N6N6N6-Trimethyl-L-lysine ↑</t>
+      <t xml:space="preserve">↓</t>
     </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">; Threonine ↑; Thr/Ser ↑</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Arginine (HMDB0000517); Citrulline (HMDB0000904); Glutamine (HMDB0000641); Threonine (HMDB0000167)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Citrullinemia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CTLN1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Citrulline ↑; N-Acetylcitrulline ↑; Arginine ↓</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Citrullinemia Type I (PathBank PW000185)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMP0000001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Citrulline (HMDB0000904); N-Acetylcitrulline (HMDB0000856); Arginine (HMDB0000517)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPT1A deficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPT1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-carnitine ↑; Palmitoylcarnitine ↓; Stearoylcarnitine ↓</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carnitine Palmitoyl Transferase Deficiency I (PathBank PW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMP0125739</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-Carnitine (HMDB0000062); Palmitoylcarnitine (HMDB0000222); Stearoylcarnitine (HMDB0000848)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPT2 deficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPT2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-carnitine ↓; Palmitoylcarnitine ↑; Oleoylcarnitine ↑;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carnitine Palmitoyl Transferase Deficiency II </t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMP0658967</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-Carnitine (HMDB0000062); Palmitoylcarnitine (HMDB0000222); Oleoylcarnitine (HMDB0005065)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cystathionine beta-synthase deficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CBS </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Methionine ↑; Glutamyl-methionine ↑; Methionine-hexose ↑; 5'-Methylthioadenosine ↑; Homocysteine ↑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cystathionine beta-Synthase Deficiency (PathBank PW000100)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMP0000177</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Methionine (HMDB0000696); Glutamyl-methionine (HMDB0034367); Methionine-hexose (no HMDB entry found); 5'-Methylthioadenosine (HMDB0001173); Homocysteine (HMDB0000742)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cytosolic phosphoenolpyruvate carboxykinase deficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">261680 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">PEPCK-C </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Glutamine ↑; Arginine ↓; Citrulline ↓ </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phosphoenolpyruvate Carboxykinase Deficiency 1 (PEPCK1) (PathBank PW000536)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMP0000560</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Glutamine (HMDB0000641); Arginine (HMDB0000517); Citrulline (HMDB0000904)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dihydropyrimidinase deficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DPH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dihydrothymine ↑; Dihydrouracil ↑; Thymine ↑; Uracil ↑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dihydropyrimidinase Deficiency (PathBank PW000189)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMP0000178</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dihydrothymine (HMDB0000079); Dihydrouracil (HMDB0000076); Thymine (HMDB0000262); Uracil (HMDB0000300)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dihydropyrimidine dehydrogenase deficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DPD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thymine ↑; Uracil ↑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dihydropyrimidine Dehydrogenase Deficiency (DHPD) (PathBank PW000198)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMP0000179</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thymine (HMDB0000262); Uracil (HMDB0000300)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dimethylglycine dehydrogenase deficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">605849 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">DMGLY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dimethylglycine ↑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dimethylglycine Dehydrogenase Deficiency (PathBank PW000197)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMP0000242</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dimethylglycine (HMDB0000092)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DNAJC12 deficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">606060 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">DNAJC12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phenylalanine ↑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phenylalanine (HMDB0000159)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ethylmalonic encephalopathy (ETHE1 deficiency)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">602473 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ETHE1 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ethylmalonic acid ↑; 2-Methylbutyrylglycine ↑; Methylsuccinic acid ↑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ethylmalonic Encephalopathy (PathBank PW000106)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMP0000181</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ethylmalonic acid (HMDB0000622); 2-Methylbutyrylglycine (HMDB0000339); Methylsuccinic acid (HMDB0001844)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Formimidoyltransferase cyclodeaminase deficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">229100 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">FIGLU </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hydantoin-5-propionic acid ↑; Formiminoglutamic acid ↑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hydantoin-5-propionic acid (HMDB0001212); Formiminoglutamic acid (HMDB0000854)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fumarate hydratase deficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">606812 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">FH1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fumaric acid ↑; Succinic acid ↑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fumarase Deficiency (PathBank PW000523)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMP0000547</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fumaric acid (HMDB0000134); Succinic acid (HMDB0000254)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Galactosemia type 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">230400 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">GAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Galactose ↑; Galactitol ↑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Galactosemia (PathBank PW000200)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMP0000182</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Galactose (HMDB0000143); Galactitol (HMDB0000107)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Glucose transporter 1 deficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GLUT1-D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Glucose ↓*; Gluconic + Galactonic acid ↓*; Xylose-α1-3-glucose ↓*; Xylose-α1-3-xylose-α1-3-glucose↓*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GLUT-1 Deficiency Syndrome (PathBank PW000556)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMP0000580</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Glucose (HMDB0000122); Gluconic + Galactonic acid (HMDB0000625; HMDB0000565); Xylose-α1-3-glucose (no HMDB entry found); Xylose-α1-3-xylose-α1-3-glucose (no HMDB entry found)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Glucose transporter 2 deficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">227810 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">FBS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fanconi-Bickel Syndrome (PathBank PW000548)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMP0000572</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Glutaric aciduria type II</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GA2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Glutaric acid ↑; Glutarylcarnitine ↑; 3-Hydroxyglutaric acid ↑; Hexanoylcarnitine ↑; Octanoylcarnitine ↑; 3, 5-Tetradecadiencarnitine ↑; cis-5-Tetradecenoylcarnitine ↑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Glutaric acid (HMDB0000661); Glutarylcarnitine (HMDB0013130); 3-Hydroxyglutaric acid (HMDB0000428); Hexanoylcarnitine (HMDB0000756); Octanoylcarnitine (HMDB0000791); 3, 5-Tetradecadiencarnitine (HMDB0241375); cis-5-Tetradecenoylcarnitine (HMDB0002014)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Glutaryl-CoA dehydrogenase deficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">231670 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">GA-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Glutaric acid ↑; Glutarylcarnitine ↑; 3-Hydroxyglutaric acid ↑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Glutaric Aciduria Type I (PathBank PW000107)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMP0000185</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Glutaric acid (HMDB0000661); Glutarylcarnitine (HMDB0013130); 3-Hydroxyglutaric acid (HMDB0000428)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guanidinoacetate methyltransferase deficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">612736 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">GAMT </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guanidinoacetic acid ↑; Creatine ↓; Creatinine ↓</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guanidinoacetate Methyltransferase Deficiency (GAMT Deficiency) (PathBank PW000088)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMP0000188</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guanidinoacetic acid (HMDB0000128); Creatine (HMDB0000064); Creatinine (HMDB0000562)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Histidine ammonia-lyase deficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">235800 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">HAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Histidine ↑; Imidazole lactic acid ↑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Histidinemia (PathBank PW000113)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMP0000191</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Histidine (HMDB0000177); Imidazole lactic acid (HMDB0002320)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Homogentisic acid oxidase deficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">203500 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">AKU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Homogentisic acid ↑; Tyrosine ↑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alkaptonuria (PathBank PW000180)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMP0000169</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Homogentisic acid (not observed in our plasma data) (HMDB0000130); Tyrosine (HMDB0000158)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hyperprolinemia type 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">239510 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">P5CDH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proline ↑; Pyrrole-2-carboxylic acid ↑; 2-Pyrroloylglycine ↑; Pyrrole-2-carboxylic acid ↑; (2 R)-5-(2-oxopropyl)pyrrolidine-2-carboxylic acid ↑; (2 R)-5-(carboxymethyl)pyrrolidine-2-carboxylic acid ↑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hyperprolinemia Type II (PathBank PW000085)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMP0000360</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proline (HMDB0000162); Pyrrole-2-carboxylic acid (HMDB0004230); 2-Pyrroloylglycine (HMDB0059778); Pyrrole-2-carboxylic acid (HMDB0004230); (2 R)-5-(2-oxopropyl)pyrrolidine-2-carboxylic acid (no HMDB entry found); (2 R)-5-(carboxymethyl)pyrrolidine-2-carboxylic acid (no HMDB entry found)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hypoxanthine guanine phosphoribosyltransferase deficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HGPRT </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hypoxanthine ↑; Xanthine ↑; Uric acid ↑; AICA riboside ↑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lesch-Nyhan Syndrome (LNS) (PathBank PW000078)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMP0000364</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hypoxanthine (HMDB0000157); Xanthine (HMDB0000292); Uric acid (HMDB0000289); AICA riboside (HMDB0062179)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Isovaleryl-CoA dehydrogenase deficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IVA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Isovalerylglycine ↑; Isovalerylcarnitine ↑; Isovaleric acid ↑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Isovaleric Aciduria (PathBank PW000091)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMP0000238</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Isovalerylglycine (HMDB0000678); Isovalerylcarnitine (HMDB0000688); Isovaleric acid (HMDB0000718)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Long-chain 3-hydroxyacyl-CoA dehydrogenase deficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LCHAD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3-Hydroxyhexadecanoylcarnitine ↑; 3-Hydroxytetradecanoylcarnitine ↑;  3-Hydroxytetradecenoylcarnitine ↑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Long-Chain-3-Hydroxyacyl-CoA Dehydrogenase Deficiency (LCHAD) (PathBank PW000520)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMP0000544</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3-Hydroxyhexadecanoylcarnitine (HMDB0013336); 3-Hydroxytetradecanoylcarnitine (HMDB0061640); 3-Hydroxytetradecenoylcarnitine (HMDB0013330)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Long-chain 3-ketoacyl CoA thiolase deficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LCKAT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hexadecanoylcarnitine ↑; 3-Hydroxyhexadecanoylcarnitine ↑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trifunctional Protein Deficiency (PathBank PW000521)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMP0000545</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hexadecanoylcarnitine (HMDB0000222); 3-Hydroxyhexadecanoylcarnitine (HMDB0013336)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lysinuric protein intolerance (LPI)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LPI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lysine ↓; Arginine ↓; Ornithine ↓; Glutamine ↑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lysinuric Protein Intolerance (LPI) (PathBank PW000561)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMP0000585</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lysine (HMDB0000182); Arginine (HMDB0000517); Ornithine (HMDB0000214); Glutamine (HMDB0000641)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Malonyl-CoA decarboxylase deficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Malonylcarnitine ↑; Malonic acid ↑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Malonyl-CoA Decarboxylase Deficiency (PathBank PW000478)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMP0000502</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Malonylcarnitine (HMDB0002095); Malonic acid (HMDB0000691)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maple syrup urine disease</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSUD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leucine ↑; Isoleucine ↑; Ketoleucine ↑; 2-Hydroxy-3-methylbutyric acid ↑; 2-Ketoisovaleric acid ↑; 3-Methyl-2-oxovaleric acid ↑; 2-Hydroxycaproic acid ↑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maple Syrup Urine Disease (PathBank PW000064)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMP0000199</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leucine (HMDB0000687); Isoleucine (HMDB0000172); Ketoleucine (HMDB0000695); 2-Hydroxy-3-methylbutyric acid (HMDB0000407); 2-Ketoisovaleric acid (HMDB0000019); 3-Methyl-2-oxovaleric acid (HMDB0000491); 2-Hydroxycaproic acid (HMDB0001624)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medium-chain acyl-CoA dehydrogenase deficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCAD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-Octanoylcarnitine ↑; Hexanoylglycine ↑; Hexanoylcarnitine ↑; 9-Decenoylcarnitine ↑; 2-trans,4-cis-Decadienoylcarnitine ↑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medium Chain Acyl-CoA Dehydrogenase Deficiency (MCAD) (PathBank PW000518)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMP0000542</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-Octanoylcarnitine (HMDB0000791); Hexanoylglycine (HMDB0000701); Hexanoylcarnitine (HMDB0000756); 9-Decenoylcarnitine (HMDB0013205); 2-trans,4-cis-Decadienoylcarnitine (HMDB0013325)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Methionine adenosyltransferase I/III deficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAT I/III </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Methionine ↑; Glutamyl-methionine ↑; Methionine-hexose ↑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Methionine Adenosyltransferase Deficiency (PathBank PW000105)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMP0000221</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Methionine (HMDB0000696); Glutamyl-methionine (HMDB0034367); Methionine-hexose (no HMDB entry found)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Methylmalonic aciduria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MMA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Methylmalonic acid ↑; Methylmalonylcarnitine ↑; Propionylcarnitine ↑; Propionic acid ↑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Methylmalonic Aciduria (PathBank PW000069)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMP0000200</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Methylmalonic acid (HMDB0000202); Methylmalonylcarnitine (HMDB0013133); Propionylcarnitine (HMDB0000824); Propionic acid (HMDB0000237)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mevalonate kinase deficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HIDS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mevalonic acid ↑; Mevalonolactone ↑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mevalonic Aciduria (PathBank PW000486)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMP0000510</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mevalonic acid (HMDB0000227); Mevalonolactone (HMDB0006024)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mitochondrial short-chain enoyl-CoA hydratase 1 deficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">616277 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ECHS1D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pyruvate ↑; 2,3-Dihydroxy-2-methylbutanoic acid ↑; S-(2-carboxypropyl)-Cysteamine ↑; S-(2-Carboxypropyl)-cysteine ↑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pyruvate (HMDB0000243); 2,3-Dihydroxy-2-methylbutanoic acid (HMDB0029576); S-(2-carboxypropyl)-Cysteamine (HMDB0002169); S-(2-Carboxypropyl)-cysteine (no HMDB entry found)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Molybdenum cofactor deficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MOCD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Xanthosine ↑; Xanthine ↑;  2,3,4,5-Tetrahydropiperidine-2-carboxylate (P6C) ↑; 4-Pyridoxic acid ↑; Uric acid ↓; Cysteine-S-sulfate ↑; L-Cystine ↓; Homocysteine ↓; Taurine ↑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Molybdenum Cofactor Deficiency (PathBank PW000079)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMP0000203</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Xanthosine (HMDB0000299); Xanthine (HMDB0000292); 2,3,4,5-Tetrahydropiperidine-2-carboxylate (P6C) (no HMDB entry found); 4-Pyridoxic acid (HMDB0000017); Uric acid (HMDB0000289); Cysteine-S-sulfate (HMDB0000731); L-Cystine (HMDB0000192); Homocysteine (HMDB0000742); Taurine (HMDB0000251)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N-acetylneuraminate pyruvate lyase deficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NPL -CDG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N-Acetylneuraminate ↑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N-Acetylneuraminate (HMDB0000230)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N-acetylneuraminic acid synthase deficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">610442 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">NANS-CDG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N-Acetylmannosamine ↑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N-Acetylmannosamine (HMDB0001129)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N-trimethyllysine hydroxylase deficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTSX6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4-Trimethylammoniobutanoic acid ↓; N6N6N6-Trimethyl-L-lysine ↑</t>
   </si>
   <si>
     <t xml:space="preserve">4-Trimethylammoniobutanoic acid (HMDB0001161); N6N6N6-Trimethyl-L-lysine (HMDB0001325)</t>
@@ -1585,9 +1595,6 @@
     <t xml:space="preserve">Sedoheptulose (HMDB0003219); Erythronic acid (HMDB0000613)</t>
   </si>
   <si>
-    <t xml:space="preserve">Trimethyllysine hydroxylase deficiency</t>
-  </si>
-  <si>
     <t xml:space="preserve">Trimethyllysine ↑; Butyrobetaine ↓</t>
   </si>
   <si>
@@ -1636,7 +1643,7 @@
     <t xml:space="preserve">VLCAD</t>
   </si>
   <si>
-    <t xml:space="preserve">3, 5-Tetradecadiencarnitine ↑; cis-5-Tetradecenoylcarnitine ↑; Tetradecanoylcarnitine ↑</t>
+    <t xml:space="preserve">3, 5-Tetradecadiencarnitine ↑; Tetradecenoylcarnitine ↑; Tetradecanoylcarnitine ↑</t>
   </si>
   <si>
     <t xml:space="preserve">Very-Long-Chain Acyl-CoA Dehydrogenase Deficiency (VLCAD) (PathBank PW000516)</t>
@@ -1645,7 +1652,7 @@
     <t xml:space="preserve">SMP0000540</t>
   </si>
   <si>
-    <t xml:space="preserve">3, 5-Tetradecadiencarnitine (HMDB0241375); cis-5-Tetradecenoylcarnitine (HMDB0002014); Tetradecanoylcarnitine (HMDB0005066)</t>
+    <t xml:space="preserve">3, 5-Tetradecadiencarnitine (HMDB0241375); Tetradecenoylcarnitine (HMDB0258884); Tetradecanoylcarnitine (HMDB0005066)</t>
   </si>
   <si>
     <t xml:space="preserve">Xanthinuria type II</t>
@@ -1700,7 +1707,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1735,6 +1742,13 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
@@ -1787,7 +1801,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1809,6 +1823,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2587,7 +2605,7 @@
       <c r="C29" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="D29" s="1" t="s">
+      <c r="D29" s="6" t="s">
         <v>164</v>
       </c>
       <c r="E29" s="1" t="s">
@@ -2710,7 +2728,7 @@
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="6" t="s">
+      <c r="A35" s="7" t="s">
         <v>195</v>
       </c>
       <c r="B35" s="2" t="n">
@@ -2742,7 +2760,7 @@
       <c r="C36" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="D36" s="6" t="s">
+      <c r="D36" s="7" t="s">
         <v>203</v>
       </c>
       <c r="E36" s="5" t="s">
@@ -2765,7 +2783,7 @@
       <c r="C37" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="D37" s="1" t="s">
+      <c r="D37" s="6" t="s">
         <v>209</v>
       </c>
       <c r="E37" s="1" t="s">
@@ -3506,7 +3524,7 @@
       <c r="C70" s="1" t="s">
         <v>407</v>
       </c>
-      <c r="D70" s="1" t="s">
+      <c r="D70" s="6" t="s">
         <v>408</v>
       </c>
       <c r="E70" s="1" t="s">
@@ -3897,7 +3915,7 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="1" t="s">
-        <v>508</v>
+        <v>406</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>300872</v>
@@ -3906,143 +3924,143 @@
         <v>407</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="E88" s="1" t="s">
         <v>36</v>
       </c>
       <c r="G88" s="1" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="1" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>276700</v>
       </c>
       <c r="C89" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="D89" s="1" t="s">
         <v>512</v>
       </c>
-      <c r="D89" s="1" t="s">
+      <c r="E89" s="1" t="s">
         <v>513</v>
       </c>
-      <c r="E89" s="1" t="s">
+      <c r="F89" s="1" t="s">
         <v>514</v>
       </c>
-      <c r="F89" s="1" t="s">
+      <c r="G89" s="1" t="s">
         <v>515</v>
-      </c>
-      <c r="G89" s="1" t="s">
-        <v>516</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="1" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>258900</v>
       </c>
       <c r="C90" s="1" t="s">
+        <v>517</v>
+      </c>
+      <c r="D90" s="1" t="s">
         <v>518</v>
       </c>
-      <c r="D90" s="1" t="s">
+      <c r="E90" s="1" t="s">
         <v>519</v>
       </c>
-      <c r="E90" s="1" t="s">
+      <c r="F90" s="1" t="s">
         <v>520</v>
       </c>
-      <c r="F90" s="1" t="s">
+      <c r="G90" s="1" t="s">
         <v>521</v>
-      </c>
-      <c r="G90" s="1" t="s">
-        <v>522</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>201475</v>
       </c>
       <c r="C91" s="1" t="s">
+        <v>523</v>
+      </c>
+      <c r="D91" s="5" t="s">
         <v>524</v>
       </c>
-      <c r="D91" s="1" t="s">
+      <c r="E91" s="1" t="s">
         <v>525</v>
       </c>
-      <c r="E91" s="1" t="s">
+      <c r="F91" s="1" t="s">
         <v>526</v>
       </c>
-      <c r="F91" s="1" t="s">
+      <c r="G91" s="5" t="s">
         <v>527</v>
-      </c>
-      <c r="G91" s="1" t="s">
-        <v>528</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="1" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>603592</v>
       </c>
       <c r="C92" s="1" t="s">
+        <v>529</v>
+      </c>
+      <c r="D92" s="1" t="s">
         <v>530</v>
       </c>
-      <c r="D92" s="1" t="s">
+      <c r="E92" s="1" t="s">
         <v>531</v>
       </c>
-      <c r="E92" s="1" t="s">
+      <c r="F92" s="1" t="s">
         <v>532</v>
       </c>
-      <c r="F92" s="1" t="s">
+      <c r="G92" s="1" t="s">
         <v>533</v>
-      </c>
-      <c r="G92" s="1" t="s">
-        <v>534</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="1" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B93" s="2" t="n">
         <v>234580</v>
       </c>
       <c r="C93" s="1" t="s">
+        <v>535</v>
+      </c>
+      <c r="D93" s="1" t="s">
         <v>536</v>
       </c>
-      <c r="D93" s="1" t="s">
+      <c r="E93" s="1" t="s">
         <v>537</v>
       </c>
-      <c r="E93" s="1" t="s">
+      <c r="F93" s="1" t="s">
         <v>538</v>
       </c>
-      <c r="F93" s="1" t="s">
+      <c r="G93" s="1" t="s">
         <v>539</v>
-      </c>
-      <c r="G93" s="1" t="s">
-        <v>540</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="1" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="1" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="1" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
     </row>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>